<commit_message>
Update RDA prompt references and enhance JSON structure in sample files
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="134">
   <si>
     <t>rda model</t>
   </si>
@@ -208,7 +208,46 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[0].type</t>
+    <t>dmp.dataset[0].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].language</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[1].dataset_id.identifier</t>
@@ -217,7 +256,28 @@
     <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[1].type</t>
+    <t>dmp.dataset[1].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[2].dataset_id.identifier</t>
@@ -226,7 +286,25 @@
     <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[2].type</t>
+    <t>dmp.dataset[2].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.dmp_id.identifier</t>
@@ -244,10 +322,7 @@
     <t>dmp.modified</t>
   </si>
   <si>
-    <t>0000-0003-0644-4174</t>
-  </si>
-  <si>
-    <t>orcid</t>
+    <t>other</t>
   </si>
   <si>
     <t>2026-10-19T00:00:00Z</t>
@@ -259,21 +334,33 @@
     <t>Data related to each of our proposed experiments</t>
   </si>
   <si>
-    <t>dataset</t>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Raw data collected from each experiment</t>
+  </si>
+  <si>
+    <t>The servers at the Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>Code for the controllers used in the experiment</t>
+  </si>
+  <si>
+    <t>eng</t>
   </si>
   <si>
     <t>Code and results for all analyses completed on experimental data</t>
   </si>
   <si>
+    <t>Code necessary to recreate figures, tables, and other results reported in all published manuscripts</t>
+  </si>
+  <si>
     <t>Simulation code for controller development and testing</t>
   </si>
   <si>
-    <t>unknown</t>
-  </si>
-  <si>
-    <t>eng</t>
-  </si>
-  <si>
     <t>CPS 2015</t>
   </si>
   <si>
@@ -283,18 +370,24 @@
     <t>data related to each of our proposed experiments</t>
   </si>
   <si>
+    <t>servers at the Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
     <t>code and results for all analyses completed on experimental data</t>
   </si>
   <si>
     <t>simulation code for controller development and testing</t>
   </si>
   <si>
+    <t>GNU Public License</t>
+  </si>
+  <si>
     <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
   </si>
   <si>
-    <t>servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
     <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
   </si>
   <si>
@@ -307,9 +400,6 @@
     <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
   </si>
   <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
     <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
@@ -322,10 +412,13 @@
     <t>Hallucinated</t>
   </si>
   <si>
+    <t>both empty</t>
+  </si>
+  <si>
     <t>not in the reference</t>
   </si>
   <si>
-    <t>both empty</t>
+    <t>empty where the reference has a value</t>
   </si>
 </sst>
 </file>
@@ -729,25 +822,25 @@
         <v>25</v>
       </c>
       <c r="D2">
+        <v>59</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2">
         <v>29</v>
       </c>
-      <c r="E2">
-        <v>20</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
       <c r="G2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>0.6899999999999999</v>
+        <v>0.508</v>
       </c>
       <c r="I2">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
       <c r="J2">
-        <v>0.506</v>
+        <v>0.514</v>
       </c>
     </row>
   </sheetData>
@@ -809,31 +902,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
+        <v>59</v>
+      </c>
+      <c r="I2">
         <v>29</v>
       </c>
-      <c r="I2">
-        <v>9</v>
-      </c>
       <c r="J2">
-        <v>0.6899999999999999</v>
+        <v>0.508</v>
       </c>
       <c r="K2">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
       <c r="L2">
-        <v>0.506</v>
+        <v>0.514</v>
       </c>
     </row>
   </sheetData>
@@ -894,7 +987,7 @@
         <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -996,7 +1089,7 @@
         <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1115,7 +1208,7 @@
         <v>46</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1295,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1337,17 +1430,14 @@
       <c r="D2" t="s">
         <v>56</v>
       </c>
-      <c r="E2" t="s">
-        <v>75</v>
-      </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1364,16 +1454,16 @@
         <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1390,13 +1480,13 @@
         <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G4" t="s">
         <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1413,13 +1503,13 @@
         <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G5" t="s">
         <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1436,16 +1526,16 @@
         <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H6" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1462,13 +1552,13 @@
         <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G7" t="s">
         <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1484,14 +1574,17 @@
       <c r="D8" t="s">
         <v>62</v>
       </c>
+      <c r="E8" t="s">
+        <v>101</v>
+      </c>
       <c r="F8" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1508,10 +1601,10 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
         <v>50</v>
@@ -1531,10 +1624,10 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="G10" t="s">
         <v>50</v>
@@ -1554,10 +1647,10 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="G11" t="s">
         <v>50</v>
@@ -1577,16 +1670,16 @@
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="F12" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G12" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H12" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1602,14 +1695,17 @@
       <c r="D13" t="s">
         <v>64</v>
       </c>
+      <c r="E13" t="s">
+        <v>106</v>
+      </c>
       <c r="F13" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="H13" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1620,19 +1716,19 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>18</v>
+      </c>
+      <c r="E14" t="s">
+        <v>107</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="G14" t="s">
         <v>50</v>
-      </c>
-      <c r="H14" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1643,19 +1739,19 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="G15" t="s">
         <v>50</v>
+      </c>
+      <c r="H15" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1666,19 +1762,19 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="G16" t="s">
         <v>50</v>
+      </c>
+      <c r="H16" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1689,19 +1785,22 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>130</v>
+      </c>
+      <c r="H17" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1712,22 +1811,22 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G18" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H18" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1738,19 +1837,22 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="E19" t="s">
+        <v>109</v>
       </c>
       <c r="F19" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G19" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1761,19 +1863,22 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
+        <v>70</v>
+      </c>
+      <c r="E20" t="s">
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="H20" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1784,19 +1889,19 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="G21" t="s">
         <v>50</v>
+      </c>
+      <c r="H21" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1807,19 +1912,19 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F22" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="G22" t="s">
         <v>50</v>
+      </c>
+      <c r="H22" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1830,19 +1935,22 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="E23" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="F23" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="G23" t="s">
-        <v>50</v>
+        <v>130</v>
+      </c>
+      <c r="H23" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1853,22 +1961,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="F24" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G24" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H24" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1879,19 +1987,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F25" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G25" t="s">
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1902,19 +2010,22 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="E26" t="s">
+        <v>101</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G26" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="H26" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1925,22 +2036,19 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
-      </c>
-      <c r="E27" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G27" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H27" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1951,22 +2059,22 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E28" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="G28" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="H28" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1977,22 +2085,19 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="D29" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="F29" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="G29" t="s">
-        <v>100</v>
-      </c>
-      <c r="H29" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2003,16 +2108,16 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D30" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="E30" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="F30" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="G30" t="s">
         <v>50</v>
@@ -2026,16 +2131,19 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>28</v>
       </c>
       <c r="E31" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="F31" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="G31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2046,275 +2154,947 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>79</v>
+      </c>
+      <c r="D32" t="s">
+        <v>79</v>
       </c>
       <c r="E32" t="s">
+        <v>105</v>
+      </c>
+      <c r="F32" t="s">
+        <v>115</v>
+      </c>
+      <c r="G32" t="s">
+        <v>130</v>
+      </c>
+      <c r="H32" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" t="s">
+        <v>112</v>
+      </c>
+      <c r="F33" t="s">
+        <v>115</v>
+      </c>
+      <c r="G33" t="s">
+        <v>130</v>
+      </c>
+      <c r="H33" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" t="s">
+        <v>81</v>
+      </c>
+      <c r="E34" t="s">
+        <v>107</v>
+      </c>
+      <c r="F34" t="s">
+        <v>118</v>
+      </c>
+      <c r="G34" t="s">
+        <v>130</v>
+      </c>
+      <c r="H34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>82</v>
+      </c>
+      <c r="D35" t="s">
+        <v>82</v>
+      </c>
+      <c r="F35" t="s">
+        <v>115</v>
+      </c>
+      <c r="G35" t="s">
+        <v>50</v>
+      </c>
+      <c r="H35" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>83</v>
+      </c>
+      <c r="D36" t="s">
+        <v>83</v>
+      </c>
+      <c r="F36" t="s">
+        <v>115</v>
+      </c>
+      <c r="G36" t="s">
+        <v>50</v>
+      </c>
+      <c r="H36" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" t="s">
+        <v>84</v>
+      </c>
+      <c r="D37" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" t="s">
+        <v>108</v>
+      </c>
+      <c r="F37" t="s">
+        <v>115</v>
+      </c>
+      <c r="G37" t="s">
+        <v>130</v>
+      </c>
+      <c r="H37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38">
+        <v>3</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" t="s">
+        <v>110</v>
+      </c>
+      <c r="F38" t="s">
+        <v>110</v>
+      </c>
+      <c r="G38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39">
+        <v>3</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" t="s">
+        <v>85</v>
+      </c>
+      <c r="D39" t="s">
+        <v>85</v>
+      </c>
+      <c r="F39" t="s">
+        <v>115</v>
+      </c>
+      <c r="G39" t="s">
+        <v>50</v>
+      </c>
+      <c r="H39" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40">
+        <v>3</v>
+      </c>
+      <c r="B40" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" t="s">
         <v>86</v>
       </c>
-      <c r="F32" t="s">
+      <c r="D40" t="s">
+        <v>86</v>
+      </c>
+      <c r="E40" t="s">
+        <v>101</v>
+      </c>
+      <c r="F40" t="s">
+        <v>115</v>
+      </c>
+      <c r="G40" t="s">
+        <v>130</v>
+      </c>
+      <c r="H40" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41">
+        <v>3</v>
+      </c>
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" t="s">
+        <v>87</v>
+      </c>
+      <c r="D41" t="s">
+        <v>87</v>
+      </c>
+      <c r="F41" t="s">
+        <v>115</v>
+      </c>
+      <c r="G41" t="s">
+        <v>50</v>
+      </c>
+      <c r="H41" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42">
+        <v>3</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" t="s">
+        <v>88</v>
+      </c>
+      <c r="E42" t="s">
+        <v>101</v>
+      </c>
+      <c r="F42" t="s">
+        <v>115</v>
+      </c>
+      <c r="G42" t="s">
+        <v>130</v>
+      </c>
+      <c r="H42" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43">
+        <v>3</v>
+      </c>
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D43" t="s">
+        <v>32</v>
+      </c>
+      <c r="E43" t="s">
+        <v>103</v>
+      </c>
+      <c r="F43" t="s">
+        <v>103</v>
+      </c>
+      <c r="G43" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44">
+        <v>3</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>33</v>
+      </c>
+      <c r="D44" t="s">
+        <v>33</v>
+      </c>
+      <c r="E44" t="s">
+        <v>103</v>
+      </c>
+      <c r="F44" t="s">
+        <v>103</v>
+      </c>
+      <c r="G44" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45">
+        <v>3</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" t="s">
+        <v>34</v>
+      </c>
+      <c r="D45" t="s">
+        <v>34</v>
+      </c>
+      <c r="E45" t="s">
+        <v>113</v>
+      </c>
+      <c r="F45" t="s">
+        <v>120</v>
+      </c>
+      <c r="G45" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46">
+        <v>3</v>
+      </c>
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" t="s">
+        <v>89</v>
+      </c>
+      <c r="D46" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" t="s">
+        <v>105</v>
+      </c>
+      <c r="F46" t="s">
+        <v>115</v>
+      </c>
+      <c r="G46" t="s">
+        <v>130</v>
+      </c>
+      <c r="H46" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47">
+        <v>3</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" t="s">
+        <v>90</v>
+      </c>
+      <c r="D47" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" t="s">
+        <v>113</v>
+      </c>
+      <c r="F47" t="s">
+        <v>115</v>
+      </c>
+      <c r="G47" t="s">
+        <v>130</v>
+      </c>
+      <c r="H47" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
         <v>91</v>
       </c>
-      <c r="G32" t="s">
+      <c r="D48" t="s">
+        <v>91</v>
+      </c>
+      <c r="E48" t="s">
+        <v>107</v>
+      </c>
+      <c r="F48" t="s">
+        <v>118</v>
+      </c>
+      <c r="G48" t="s">
+        <v>130</v>
+      </c>
+      <c r="H48" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>92</v>
+      </c>
+      <c r="D49" t="s">
+        <v>92</v>
+      </c>
+      <c r="F49" t="s">
+        <v>115</v>
+      </c>
+      <c r="G49" t="s">
+        <v>50</v>
+      </c>
+      <c r="H49" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>30</v>
+      </c>
+      <c r="D50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F50" t="s">
+        <v>121</v>
+      </c>
+      <c r="G50" t="s">
+        <v>130</v>
+      </c>
+      <c r="H50" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>93</v>
+      </c>
+      <c r="D51" t="s">
+        <v>93</v>
+      </c>
+      <c r="E51" t="s">
+        <v>108</v>
+      </c>
+      <c r="F51" t="s">
+        <v>115</v>
+      </c>
+      <c r="G51" t="s">
+        <v>130</v>
+      </c>
+      <c r="H51" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>31</v>
+      </c>
+      <c r="D52" t="s">
+        <v>31</v>
+      </c>
+      <c r="E52" t="s">
+        <v>110</v>
+      </c>
+      <c r="F52" t="s">
+        <v>110</v>
+      </c>
+      <c r="G52" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53" t="s">
+        <v>115</v>
+      </c>
+      <c r="G53" t="s">
+        <v>50</v>
+      </c>
+      <c r="H53" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>95</v>
+      </c>
+      <c r="D54" t="s">
+        <v>95</v>
+      </c>
+      <c r="E54" t="s">
+        <v>101</v>
+      </c>
+      <c r="F54" t="s">
+        <v>115</v>
+      </c>
+      <c r="G54" t="s">
+        <v>130</v>
+      </c>
+      <c r="H54" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" t="s">
+        <v>96</v>
+      </c>
+      <c r="D55" t="s">
+        <v>96</v>
+      </c>
+      <c r="F55" t="s">
+        <v>115</v>
+      </c>
+      <c r="G55" t="s">
+        <v>50</v>
+      </c>
+      <c r="H55" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>97</v>
+      </c>
+      <c r="D56" t="s">
+        <v>97</v>
+      </c>
+      <c r="E56" t="s">
+        <v>101</v>
+      </c>
+      <c r="F56" t="s">
+        <v>115</v>
+      </c>
+      <c r="G56" t="s">
+        <v>130</v>
+      </c>
+      <c r="H56" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
+        <v>98</v>
+      </c>
+      <c r="D57" t="s">
+        <v>98</v>
+      </c>
+      <c r="E57" t="s">
+        <v>103</v>
+      </c>
+      <c r="F57" t="s">
+        <v>115</v>
+      </c>
+      <c r="G57" t="s">
+        <v>130</v>
+      </c>
+      <c r="H57" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58">
+        <v>3</v>
+      </c>
+      <c r="B58" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" t="s">
+        <v>99</v>
+      </c>
+      <c r="D58" t="s">
+        <v>99</v>
+      </c>
+      <c r="E58" t="s">
+        <v>110</v>
+      </c>
+      <c r="F58" t="s">
+        <v>115</v>
+      </c>
+      <c r="G58" t="s">
+        <v>130</v>
+      </c>
+      <c r="H58" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" t="s">
+        <v>100</v>
+      </c>
+      <c r="D59" t="s">
+        <v>100</v>
+      </c>
+      <c r="E59" t="s">
+        <v>102</v>
+      </c>
+      <c r="F59" t="s">
+        <v>115</v>
+      </c>
+      <c r="G59" t="s">
+        <v>130</v>
+      </c>
+      <c r="H59" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" t="s">
+        <v>41</v>
+      </c>
+      <c r="D60" t="s">
+        <v>41</v>
+      </c>
+      <c r="E60" t="s">
+        <v>114</v>
+      </c>
+      <c r="F60" t="s">
+        <v>114</v>
+      </c>
+      <c r="G60" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61">
+        <v>3</v>
+      </c>
+      <c r="B61" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" t="s">
+        <v>17</v>
+      </c>
+      <c r="E61" t="s">
+        <v>115</v>
+      </c>
+      <c r="F61" t="s">
+        <v>122</v>
+      </c>
+      <c r="G61" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
-      <c r="A33">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" t="s">
+    <row r="62" spans="1:8">
+      <c r="A62">
+        <v>3</v>
+      </c>
+      <c r="B62" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" t="s">
         <v>22</v>
       </c>
-      <c r="E33" t="s">
-        <v>86</v>
-      </c>
-      <c r="F33" t="s">
-        <v>92</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="E62" t="s">
+        <v>115</v>
+      </c>
+      <c r="F62" t="s">
+        <v>123</v>
+      </c>
+      <c r="G62" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
-      <c r="A34">
-        <v>3</v>
-      </c>
-      <c r="B34" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" t="s">
+    <row r="63" spans="1:8">
+      <c r="A63">
+        <v>3</v>
+      </c>
+      <c r="B63" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" t="s">
         <v>23</v>
       </c>
-      <c r="E34" t="s">
-        <v>86</v>
-      </c>
-      <c r="F34" t="s">
-        <v>93</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="E63" t="s">
+        <v>115</v>
+      </c>
+      <c r="F63" t="s">
+        <v>124</v>
+      </c>
+      <c r="G63" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
-      <c r="A35">
-        <v>3</v>
-      </c>
-      <c r="B35" t="s">
-        <v>10</v>
-      </c>
-      <c r="C35" t="s">
-        <v>24</v>
-      </c>
-      <c r="E35" t="s">
-        <v>86</v>
-      </c>
-      <c r="F35" t="s">
-        <v>84</v>
-      </c>
-      <c r="G35" t="s">
+    <row r="64" spans="1:8">
+      <c r="A64">
+        <v>3</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" t="s">
+        <v>25</v>
+      </c>
+      <c r="E64" t="s">
+        <v>115</v>
+      </c>
+      <c r="F64" t="s">
+        <v>125</v>
+      </c>
+      <c r="G64" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
-      <c r="A36">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
-        <v>10</v>
-      </c>
-      <c r="C36" t="s">
-        <v>25</v>
-      </c>
-      <c r="E36" t="s">
-        <v>86</v>
-      </c>
-      <c r="F36" t="s">
-        <v>94</v>
-      </c>
-      <c r="G36" t="s">
+    <row r="65" spans="1:7">
+      <c r="A65">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
+        <v>29</v>
+      </c>
+      <c r="E65" t="s">
+        <v>115</v>
+      </c>
+      <c r="F65" t="s">
+        <v>126</v>
+      </c>
+      <c r="G65" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
-      <c r="A37">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" t="s">
-        <v>86</v>
-      </c>
-      <c r="F37" t="s">
-        <v>95</v>
-      </c>
-      <c r="G37" t="s">
+    <row r="66" spans="1:7">
+      <c r="A66">
+        <v>3</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>30</v>
+      </c>
+      <c r="E66" t="s">
+        <v>115</v>
+      </c>
+      <c r="F66" t="s">
+        <v>121</v>
+      </c>
+      <c r="G66" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
-      <c r="A38">
-        <v>3</v>
-      </c>
-      <c r="B38" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" t="s">
-        <v>30</v>
-      </c>
-      <c r="E38" t="s">
-        <v>86</v>
-      </c>
-      <c r="F38" t="s">
-        <v>96</v>
-      </c>
-      <c r="G38" t="s">
+    <row r="67" spans="1:7">
+      <c r="A67">
+        <v>3</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>35</v>
+      </c>
+      <c r="E67" t="s">
+        <v>115</v>
+      </c>
+      <c r="F67" t="s">
+        <v>127</v>
+      </c>
+      <c r="G67" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
-      <c r="A39">
-        <v>3</v>
-      </c>
-      <c r="B39" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" t="s">
-        <v>31</v>
-      </c>
-      <c r="E39" t="s">
-        <v>86</v>
-      </c>
-      <c r="F39" t="s">
-        <v>84</v>
-      </c>
-      <c r="G39" t="s">
+    <row r="68" spans="1:7">
+      <c r="A68">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" t="s">
+        <v>36</v>
+      </c>
+      <c r="E68" t="s">
+        <v>115</v>
+      </c>
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
-      <c r="A40">
-        <v>3</v>
-      </c>
-      <c r="B40" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" t="s">
-        <v>35</v>
-      </c>
-      <c r="E40" t="s">
-        <v>86</v>
-      </c>
-      <c r="F40" t="s">
-        <v>97</v>
-      </c>
-      <c r="G40" t="s">
+    <row r="69" spans="1:7">
+      <c r="A69">
+        <v>3</v>
+      </c>
+      <c r="B69" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
+        <v>37</v>
+      </c>
+      <c r="E69" t="s">
+        <v>115</v>
+      </c>
+      <c r="F69" t="s">
+        <v>103</v>
+      </c>
+      <c r="G69" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
-      <c r="A41">
-        <v>3</v>
-      </c>
-      <c r="B41" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" t="s">
-        <v>36</v>
-      </c>
-      <c r="E41" t="s">
-        <v>86</v>
-      </c>
-      <c r="F41" t="s">
-        <v>84</v>
-      </c>
-      <c r="G41" t="s">
+    <row r="70" spans="1:7">
+      <c r="A70">
+        <v>3</v>
+      </c>
+      <c r="B70" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" t="s">
+        <v>38</v>
+      </c>
+      <c r="E70" t="s">
+        <v>115</v>
+      </c>
+      <c r="F70" t="s">
+        <v>103</v>
+      </c>
+      <c r="G70" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
-      <c r="A42">
-        <v>3</v>
-      </c>
-      <c r="B42" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" t="s">
-        <v>37</v>
-      </c>
-      <c r="E42" t="s">
-        <v>86</v>
-      </c>
-      <c r="F42" t="s">
-        <v>78</v>
-      </c>
-      <c r="G42" t="s">
+    <row r="71" spans="1:7">
+      <c r="A71">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" t="s">
+        <v>39</v>
+      </c>
+      <c r="E71" t="s">
+        <v>115</v>
+      </c>
+      <c r="F71" t="s">
+        <v>128</v>
+      </c>
+      <c r="G71" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="B43" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" t="s">
-        <v>38</v>
-      </c>
-      <c r="E43" t="s">
-        <v>86</v>
-      </c>
-      <c r="F43" t="s">
-        <v>78</v>
-      </c>
-      <c r="G43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44">
-        <v>3</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s">
-        <v>39</v>
-      </c>
-      <c r="E44" t="s">
-        <v>86</v>
-      </c>
-      <c r="F44" t="s">
-        <v>98</v>
-      </c>
-      <c r="G44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45">
-        <v>3</v>
-      </c>
-      <c r="B45" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" t="s">
+    <row r="72" spans="1:7">
+      <c r="A72">
+        <v>3</v>
+      </c>
+      <c r="B72" t="s">
+        <v>10</v>
+      </c>
+      <c r="C72" t="s">
         <v>40</v>
       </c>
-      <c r="E45" t="s">
-        <v>86</v>
-      </c>
-      <c r="F45" t="s">
-        <v>99</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="E72" t="s">
+        <v>115</v>
+      </c>
+      <c r="F72" t="s">
+        <v>129</v>
+      </c>
+      <c r="G72" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RDA narrative prompt to version 10d and adjust related notebook configurations
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="111">
   <si>
     <t>rda model</t>
   </si>
@@ -208,46 +208,7 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[0].distribution[0].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[0].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[0].host.url</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].host.title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].host.url</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].metadata[0].language</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].type</t>
+    <t>dmp.dataset[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[1].dataset_id.identifier</t>
@@ -256,28 +217,7 @@
     <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[1].distribution[0].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].host.title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].host.url</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].type</t>
+    <t>dmp.dataset[1].type</t>
   </si>
   <si>
     <t>dmp.dataset[2].dataset_id.identifier</t>
@@ -286,25 +226,7 @@
     <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[2].distribution[0].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].distribution[0].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].distribution[0].host.title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].distribution[0].host.url</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].type</t>
+    <t>dmp.dataset[2].type</t>
   </si>
   <si>
     <t>dmp.dmp_id.identifier</t>
@@ -322,6 +244,30 @@
     <t>dmp.modified</t>
   </si>
   <si>
+    <t>dmp.project[0].title</t>
+  </si>
+  <si>
+    <t>dmp.project[0].description</t>
+  </si>
+  <si>
+    <t>dmp.project[0].funding[0].funder_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.project[0].funding[0].funder_id.type</t>
+  </si>
+  <si>
+    <t>dmp.project[0].funding[0].funding_status</t>
+  </si>
+  <si>
+    <t>dmp.related_identifier[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.related_identifier[0].relation_type</t>
+  </si>
+  <si>
+    <t>dmp.related_identifier[0].type</t>
+  </si>
+  <si>
     <t>other</t>
   </si>
   <si>
@@ -334,72 +280,60 @@
     <t>Data related to each of our proposed experiments</t>
   </si>
   <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>Raw data collected from each experiment</t>
-  </si>
-  <si>
-    <t>The servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>Code for the controllers used in the experiment</t>
+    <t>dataset</t>
+  </si>
+  <si>
+    <t>Code and results for all analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>Simulation code for controller development and testing</t>
   </si>
   <si>
     <t>eng</t>
   </si>
   <si>
-    <t>Code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>Code necessary to recreate figures, tables, and other results reported in all published manuscripts</t>
-  </si>
-  <si>
-    <t>Simulation code for controller development and testing</t>
-  </si>
-  <si>
     <t>CPS 2015</t>
   </si>
   <si>
+    <t>The project aims to manage and disseminate data generated by the project.</t>
+  </si>
+  <si>
+    <t>planned</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
     <t>data related to each of our proposed experiments</t>
   </si>
   <si>
+    <t>code and results for all analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>simulation code for controller development and testing</t>
+  </si>
+  <si>
+    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
     <t>servers at the Rehabilitation Institute of Chicago</t>
   </si>
   <si>
-    <t>null</t>
-  </si>
-  <si>
-    <t>code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>simulation code for controller development and testing</t>
+    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+  </si>
+  <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+  </si>
+  <si>
+    <t>The code needed to generate all published results will be documented clearly.</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
   </si>
   <si>
     <t>GNU Public License</t>
   </si>
   <si>
-    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
-  </si>
-  <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
-  </si>
-  <si>
-    <t>The code needed to generate all published results will be documented clearly.</t>
-  </si>
-  <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
     <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
@@ -416,9 +350,6 @@
   </si>
   <si>
     <t>not in the reference</t>
-  </si>
-  <si>
-    <t>empty where the reference has a value</t>
   </si>
 </sst>
 </file>
@@ -822,25 +753,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="E2">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H2">
-        <v>0.508</v>
+        <v>0.514</v>
       </c>
       <c r="I2">
-        <v>0.52</v>
+        <v>0.4</v>
       </c>
       <c r="J2">
-        <v>0.514</v>
+        <v>0.45</v>
       </c>
     </row>
   </sheetData>
@@ -902,31 +833,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="I2">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="J2">
-        <v>0.508</v>
+        <v>0.514</v>
       </c>
       <c r="K2">
-        <v>0.52</v>
+        <v>0.4</v>
       </c>
       <c r="L2">
-        <v>0.514</v>
+        <v>0.45</v>
       </c>
     </row>
   </sheetData>
@@ -987,7 +918,7 @@
         <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1089,7 +1020,7 @@
         <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1208,7 +1139,7 @@
         <v>46</v>
       </c>
       <c r="E16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1388,7 +1319,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1431,13 +1362,13 @@
         <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
         <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1454,16 +1385,16 @@
         <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G3" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H3" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1480,13 +1411,13 @@
         <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G4" t="s">
         <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1503,13 +1434,13 @@
         <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G5" t="s">
         <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1526,16 +1457,16 @@
         <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G6" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H6" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1552,13 +1483,13 @@
         <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G7" t="s">
         <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1575,16 +1506,16 @@
         <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="F8" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G8" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H8" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1601,10 +1532,10 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
         <v>50</v>
@@ -1624,10 +1555,10 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G10" t="s">
         <v>50</v>
@@ -1647,10 +1578,10 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="F11" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="G11" t="s">
         <v>50</v>
@@ -1670,16 +1601,16 @@
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G12" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H12" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1695,17 +1626,14 @@
       <c r="D13" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s">
-        <v>106</v>
-      </c>
       <c r="F13" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1716,19 +1644,22 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>108</v>
+      </c>
+      <c r="H14" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1739,19 +1670,19 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>26</v>
+      </c>
+      <c r="E15" t="s">
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="G15" t="s">
         <v>50</v>
-      </c>
-      <c r="H15" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1762,19 +1693,19 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="G16" t="s">
         <v>50</v>
-      </c>
-      <c r="H16" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1785,22 +1716,19 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="G17" t="s">
-        <v>130</v>
-      </c>
-      <c r="H17" t="s">
-        <v>132</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1811,22 +1739,22 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H18" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1837,22 +1765,19 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" t="s">
         <v>109</v>
-      </c>
-      <c r="F19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" t="s">
-        <v>130</v>
-      </c>
-      <c r="H19" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1863,22 +1788,22 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E20" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="G20" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H20" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1889,19 +1814,19 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>32</v>
+      </c>
+      <c r="E21" t="s">
+        <v>85</v>
       </c>
       <c r="F21" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="G21" t="s">
         <v>50</v>
-      </c>
-      <c r="H21" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1912,19 +1837,19 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>33</v>
+      </c>
+      <c r="E22" t="s">
+        <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="G22" t="s">
         <v>50</v>
-      </c>
-      <c r="H22" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1935,22 +1860,19 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="D23" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="F23" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="G23" t="s">
-        <v>130</v>
-      </c>
-      <c r="H23" t="s">
-        <v>132</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1961,22 +1883,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
+        <v>87</v>
+      </c>
+      <c r="F24" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" t="s">
         <v>110</v>
-      </c>
-      <c r="F24" t="s">
-        <v>115</v>
-      </c>
-      <c r="G24" t="s">
-        <v>130</v>
-      </c>
-      <c r="H24" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1987,19 +1909,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D25" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G25" t="s">
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2010,22 +1932,22 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E26" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="F26" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H26" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2036,19 +1958,22 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D27" t="s">
-        <v>77</v>
+        <v>72</v>
+      </c>
+      <c r="E27" t="s">
+        <v>85</v>
       </c>
       <c r="F27" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G27" t="s">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="H27" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2059,22 +1984,22 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F28" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G28" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H28" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2085,19 +2010,22 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="E29" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="F29" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="G29" t="s">
-        <v>50</v>
+        <v>108</v>
+      </c>
+      <c r="H29" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2108,16 +2036,16 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="D30" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E30" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="F30" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="G30" t="s">
         <v>50</v>
@@ -2131,19 +2059,22 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="E31" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="F31" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="G31" t="s">
-        <v>50</v>
+        <v>108</v>
+      </c>
+      <c r="H31" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2154,22 +2085,22 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E32" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="F32" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G32" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H32" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2180,22 +2111,19 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D33" t="s">
-        <v>80</v>
-      </c>
-      <c r="E33" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="F33" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G33" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="H33" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2206,22 +2134,22 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E34" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="F34" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="G34" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="H34" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2232,19 +2160,22 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>82</v>
+        <v>79</v>
+      </c>
+      <c r="E35" t="s">
+        <v>93</v>
       </c>
       <c r="F35" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G35" t="s">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="H35" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2255,19 +2186,19 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D36" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F36" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="G36" t="s">
         <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2278,22 +2209,22 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D37" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" t="s">
+        <v>94</v>
+      </c>
+      <c r="G37" t="s">
         <v>108</v>
       </c>
-      <c r="F37" t="s">
-        <v>115</v>
-      </c>
-      <c r="G37" t="s">
-        <v>130</v>
-      </c>
       <c r="H37" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2304,19 +2235,22 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="D38" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="E38" t="s">
+        <v>83</v>
+      </c>
+      <c r="F38" t="s">
+        <v>94</v>
+      </c>
+      <c r="G38" t="s">
+        <v>108</v>
+      </c>
+      <c r="H38" t="s">
         <v>110</v>
-      </c>
-      <c r="F38" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2327,19 +2261,16 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>85</v>
-      </c>
-      <c r="D39" t="s">
-        <v>85</v>
+        <v>17</v>
+      </c>
+      <c r="E39" t="s">
+        <v>94</v>
       </c>
       <c r="F39" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="G39" t="s">
-        <v>50</v>
-      </c>
-      <c r="H39" t="s">
-        <v>131</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2350,22 +2281,16 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>86</v>
-      </c>
-      <c r="D40" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E40" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="F40" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="G40" t="s">
-        <v>130</v>
-      </c>
-      <c r="H40" t="s">
-        <v>132</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2376,19 +2301,16 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>87</v>
-      </c>
-      <c r="D41" t="s">
-        <v>87</v>
+        <v>22</v>
+      </c>
+      <c r="E41" t="s">
+        <v>94</v>
       </c>
       <c r="F41" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G41" t="s">
-        <v>50</v>
-      </c>
-      <c r="H41" t="s">
-        <v>131</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2399,22 +2321,16 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>88</v>
-      </c>
-      <c r="D42" t="s">
-        <v>88</v>
+        <v>23</v>
       </c>
       <c r="E42" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42" t="s">
         <v>101</v>
       </c>
-      <c r="F42" t="s">
-        <v>115</v>
-      </c>
       <c r="G42" t="s">
-        <v>130</v>
-      </c>
-      <c r="H42" t="s">
-        <v>132</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2425,19 +2341,16 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>32</v>
-      </c>
-      <c r="D43" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E43" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F43" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="G43" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2448,19 +2361,16 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>33</v>
-      </c>
-      <c r="D44" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F44" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2471,19 +2381,16 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>34</v>
-      </c>
-      <c r="D45" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E45" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="F45" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="G45" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2494,22 +2401,16 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>89</v>
-      </c>
-      <c r="D46" t="s">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="E46" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F46" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G46" t="s">
-        <v>130</v>
-      </c>
-      <c r="H46" t="s">
-        <v>132</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2520,22 +2421,16 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="E47" t="s">
+        <v>94</v>
+      </c>
+      <c r="F47" t="s">
         <v>90</v>
       </c>
-      <c r="D47" t="s">
-        <v>90</v>
-      </c>
-      <c r="E47" t="s">
-        <v>113</v>
-      </c>
-      <c r="F47" t="s">
-        <v>115</v>
-      </c>
       <c r="G47" t="s">
-        <v>130</v>
-      </c>
-      <c r="H47" t="s">
-        <v>132</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2546,555 +2441,115 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>91</v>
-      </c>
-      <c r="D48" t="s">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="E48" t="s">
+        <v>94</v>
+      </c>
+      <c r="F48" t="s">
+        <v>105</v>
+      </c>
+      <c r="G48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>36</v>
+      </c>
+      <c r="E49" t="s">
+        <v>94</v>
+      </c>
+      <c r="F49" t="s">
+        <v>90</v>
+      </c>
+      <c r="G49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>37</v>
+      </c>
+      <c r="E50" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50" t="s">
+        <v>85</v>
+      </c>
+      <c r="G50" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>38</v>
+      </c>
+      <c r="E51" t="s">
+        <v>94</v>
+      </c>
+      <c r="F51" t="s">
+        <v>85</v>
+      </c>
+      <c r="G51" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>39</v>
+      </c>
+      <c r="E52" t="s">
+        <v>94</v>
+      </c>
+      <c r="F52" t="s">
+        <v>106</v>
+      </c>
+      <c r="G52" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>40</v>
+      </c>
+      <c r="E53" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53" t="s">
         <v>107</v>
       </c>
-      <c r="F48" t="s">
-        <v>118</v>
-      </c>
-      <c r="G48" t="s">
-        <v>130</v>
-      </c>
-      <c r="H48" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49">
-        <v>3</v>
-      </c>
-      <c r="B49" t="s">
-        <v>10</v>
-      </c>
-      <c r="C49" t="s">
-        <v>92</v>
-      </c>
-      <c r="D49" t="s">
-        <v>92</v>
-      </c>
-      <c r="F49" t="s">
-        <v>115</v>
-      </c>
-      <c r="G49" t="s">
-        <v>50</v>
-      </c>
-      <c r="H49" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
-      <c r="A50">
-        <v>3</v>
-      </c>
-      <c r="B50" t="s">
-        <v>10</v>
-      </c>
-      <c r="C50" t="s">
-        <v>30</v>
-      </c>
-      <c r="D50" t="s">
-        <v>30</v>
-      </c>
-      <c r="F50" t="s">
-        <v>121</v>
-      </c>
-      <c r="G50" t="s">
-        <v>130</v>
-      </c>
-      <c r="H50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51">
-        <v>3</v>
-      </c>
-      <c r="B51" t="s">
-        <v>10</v>
-      </c>
-      <c r="C51" t="s">
-        <v>93</v>
-      </c>
-      <c r="D51" t="s">
-        <v>93</v>
-      </c>
-      <c r="E51" t="s">
-        <v>108</v>
-      </c>
-      <c r="F51" t="s">
-        <v>115</v>
-      </c>
-      <c r="G51" t="s">
-        <v>130</v>
-      </c>
-      <c r="H51" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
-      <c r="A52">
-        <v>3</v>
-      </c>
-      <c r="B52" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" t="s">
-        <v>31</v>
-      </c>
-      <c r="D52" t="s">
-        <v>31</v>
-      </c>
-      <c r="E52" t="s">
-        <v>110</v>
-      </c>
-      <c r="F52" t="s">
-        <v>110</v>
-      </c>
-      <c r="G52" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
-      <c r="A53">
-        <v>3</v>
-      </c>
-      <c r="B53" t="s">
-        <v>10</v>
-      </c>
-      <c r="C53" t="s">
-        <v>94</v>
-      </c>
-      <c r="D53" t="s">
-        <v>94</v>
-      </c>
-      <c r="F53" t="s">
-        <v>115</v>
-      </c>
       <c r="G53" t="s">
-        <v>50</v>
-      </c>
-      <c r="H53" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
-      <c r="A54">
-        <v>3</v>
-      </c>
-      <c r="B54" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" t="s">
-        <v>95</v>
-      </c>
-      <c r="D54" t="s">
-        <v>95</v>
-      </c>
-      <c r="E54" t="s">
-        <v>101</v>
-      </c>
-      <c r="F54" t="s">
-        <v>115</v>
-      </c>
-      <c r="G54" t="s">
-        <v>130</v>
-      </c>
-      <c r="H54" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8">
-      <c r="A55">
-        <v>3</v>
-      </c>
-      <c r="B55" t="s">
-        <v>10</v>
-      </c>
-      <c r="C55" t="s">
-        <v>96</v>
-      </c>
-      <c r="D55" t="s">
-        <v>96</v>
-      </c>
-      <c r="F55" t="s">
-        <v>115</v>
-      </c>
-      <c r="G55" t="s">
-        <v>50</v>
-      </c>
-      <c r="H55" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8">
-      <c r="A56">
-        <v>3</v>
-      </c>
-      <c r="B56" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" t="s">
-        <v>97</v>
-      </c>
-      <c r="D56" t="s">
-        <v>97</v>
-      </c>
-      <c r="E56" t="s">
-        <v>101</v>
-      </c>
-      <c r="F56" t="s">
-        <v>115</v>
-      </c>
-      <c r="G56" t="s">
-        <v>130</v>
-      </c>
-      <c r="H56" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8">
-      <c r="A57">
-        <v>3</v>
-      </c>
-      <c r="B57" t="s">
-        <v>10</v>
-      </c>
-      <c r="C57" t="s">
-        <v>98</v>
-      </c>
-      <c r="D57" t="s">
-        <v>98</v>
-      </c>
-      <c r="E57" t="s">
-        <v>103</v>
-      </c>
-      <c r="F57" t="s">
-        <v>115</v>
-      </c>
-      <c r="G57" t="s">
-        <v>130</v>
-      </c>
-      <c r="H57" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8">
-      <c r="A58">
-        <v>3</v>
-      </c>
-      <c r="B58" t="s">
-        <v>10</v>
-      </c>
-      <c r="C58" t="s">
-        <v>99</v>
-      </c>
-      <c r="D58" t="s">
-        <v>99</v>
-      </c>
-      <c r="E58" t="s">
-        <v>110</v>
-      </c>
-      <c r="F58" t="s">
-        <v>115</v>
-      </c>
-      <c r="G58" t="s">
-        <v>130</v>
-      </c>
-      <c r="H58" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8">
-      <c r="A59">
-        <v>3</v>
-      </c>
-      <c r="B59" t="s">
-        <v>10</v>
-      </c>
-      <c r="C59" t="s">
-        <v>100</v>
-      </c>
-      <c r="D59" t="s">
-        <v>100</v>
-      </c>
-      <c r="E59" t="s">
-        <v>102</v>
-      </c>
-      <c r="F59" t="s">
-        <v>115</v>
-      </c>
-      <c r="G59" t="s">
-        <v>130</v>
-      </c>
-      <c r="H59" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8">
-      <c r="A60">
-        <v>3</v>
-      </c>
-      <c r="B60" t="s">
-        <v>10</v>
-      </c>
-      <c r="C60" t="s">
-        <v>41</v>
-      </c>
-      <c r="D60" t="s">
-        <v>41</v>
-      </c>
-      <c r="E60" t="s">
-        <v>114</v>
-      </c>
-      <c r="F60" t="s">
-        <v>114</v>
-      </c>
-      <c r="G60" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
-      <c r="A61">
-        <v>3</v>
-      </c>
-      <c r="B61" t="s">
-        <v>10</v>
-      </c>
-      <c r="C61" t="s">
-        <v>17</v>
-      </c>
-      <c r="E61" t="s">
-        <v>115</v>
-      </c>
-      <c r="F61" t="s">
-        <v>122</v>
-      </c>
-      <c r="G61" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
-      <c r="A62">
-        <v>3</v>
-      </c>
-      <c r="B62" t="s">
-        <v>10</v>
-      </c>
-      <c r="C62" t="s">
-        <v>22</v>
-      </c>
-      <c r="E62" t="s">
-        <v>115</v>
-      </c>
-      <c r="F62" t="s">
-        <v>123</v>
-      </c>
-      <c r="G62" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8">
-      <c r="A63">
-        <v>3</v>
-      </c>
-      <c r="B63" t="s">
-        <v>10</v>
-      </c>
-      <c r="C63" t="s">
-        <v>23</v>
-      </c>
-      <c r="E63" t="s">
-        <v>115</v>
-      </c>
-      <c r="F63" t="s">
-        <v>124</v>
-      </c>
-      <c r="G63" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8">
-      <c r="A64">
-        <v>3</v>
-      </c>
-      <c r="B64" t="s">
-        <v>10</v>
-      </c>
-      <c r="C64" t="s">
-        <v>25</v>
-      </c>
-      <c r="E64" t="s">
-        <v>115</v>
-      </c>
-      <c r="F64" t="s">
-        <v>125</v>
-      </c>
-      <c r="G64" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7">
-      <c r="A65">
-        <v>3</v>
-      </c>
-      <c r="B65" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" t="s">
-        <v>29</v>
-      </c>
-      <c r="E65" t="s">
-        <v>115</v>
-      </c>
-      <c r="F65" t="s">
-        <v>126</v>
-      </c>
-      <c r="G65" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
-      <c r="A66">
-        <v>3</v>
-      </c>
-      <c r="B66" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" t="s">
-        <v>30</v>
-      </c>
-      <c r="E66" t="s">
-        <v>115</v>
-      </c>
-      <c r="F66" t="s">
-        <v>121</v>
-      </c>
-      <c r="G66" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
-      <c r="A67">
-        <v>3</v>
-      </c>
-      <c r="B67" t="s">
-        <v>10</v>
-      </c>
-      <c r="C67" t="s">
-        <v>35</v>
-      </c>
-      <c r="E67" t="s">
-        <v>115</v>
-      </c>
-      <c r="F67" t="s">
-        <v>127</v>
-      </c>
-      <c r="G67" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
-      <c r="A68">
-        <v>3</v>
-      </c>
-      <c r="B68" t="s">
-        <v>10</v>
-      </c>
-      <c r="C68" t="s">
-        <v>36</v>
-      </c>
-      <c r="E68" t="s">
-        <v>115</v>
-      </c>
-      <c r="F68" t="s">
-        <v>110</v>
-      </c>
-      <c r="G68" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69">
-        <v>3</v>
-      </c>
-      <c r="B69" t="s">
-        <v>10</v>
-      </c>
-      <c r="C69" t="s">
-        <v>37</v>
-      </c>
-      <c r="E69" t="s">
-        <v>115</v>
-      </c>
-      <c r="F69" t="s">
-        <v>103</v>
-      </c>
-      <c r="G69" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70">
-        <v>3</v>
-      </c>
-      <c r="B70" t="s">
-        <v>10</v>
-      </c>
-      <c r="C70" t="s">
-        <v>38</v>
-      </c>
-      <c r="E70" t="s">
-        <v>115</v>
-      </c>
-      <c r="F70" t="s">
-        <v>103</v>
-      </c>
-      <c r="G70" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
-      <c r="A71">
-        <v>3</v>
-      </c>
-      <c r="B71" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" t="s">
-        <v>39</v>
-      </c>
-      <c r="E71" t="s">
-        <v>115</v>
-      </c>
-      <c r="F71" t="s">
-        <v>128</v>
-      </c>
-      <c r="G71" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7">
-      <c r="A72">
-        <v>3</v>
-      </c>
-      <c r="B72" t="s">
-        <v>10</v>
-      </c>
-      <c r="C72" t="s">
-        <v>40</v>
-      </c>
-      <c r="E72" t="s">
-        <v>115</v>
-      </c>
-      <c r="F72" t="s">
-        <v>129</v>
-      </c>
-      <c r="G72" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance RDA maDMP JSON schema with additional dataset entries and update prompt handling
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="118">
   <si>
     <t>rda model</t>
   </si>
@@ -172,6 +172,9 @@
     <t>Correct</t>
   </si>
   <si>
+    <t>Mismatch</t>
+  </si>
+  <si>
     <t>model field</t>
   </si>
   <si>
@@ -229,6 +232,15 @@
     <t>dmp.dataset[2].type</t>
   </si>
   <si>
+    <t>dmp.dataset[3].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].dataset_id.type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].type</t>
+  </si>
+  <si>
     <t>dmp.dmp_id.identifier</t>
   </si>
   <si>
@@ -289,6 +301,9 @@
     <t>Simulation code for controller development and testing</t>
   </si>
   <si>
+    <t>Software generated under the project</t>
+  </si>
+  <si>
     <t>eng</t>
   </si>
   <si>
@@ -301,6 +316,9 @@
     <t>planned</t>
   </si>
   <si>
+    <t>isPartOf</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
@@ -313,6 +331,9 @@
     <t>simulation code for controller development and testing</t>
   </si>
   <si>
+    <t>videos of the experiments</t>
+  </si>
+  <si>
     <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
   </si>
   <si>
@@ -337,9 +358,6 @@
     <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
-    <t>videos of the experiments</t>
-  </si>
-  <si>
     <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
   </si>
   <si>
@@ -350,6 +368,9 @@
   </si>
   <si>
     <t>not in the reference</t>
+  </si>
+  <si>
+    <t>only 20% of the model's words are in the reference</t>
   </si>
 </sst>
 </file>
@@ -753,25 +774,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H2">
-        <v>0.514</v>
+        <v>0.512</v>
       </c>
       <c r="I2">
-        <v>0.4</v>
+        <v>0.48</v>
       </c>
       <c r="J2">
-        <v>0.45</v>
+        <v>0.495</v>
       </c>
     </row>
   </sheetData>
@@ -833,31 +854,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="I2">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J2">
-        <v>0.514</v>
+        <v>0.512</v>
       </c>
       <c r="K2">
-        <v>0.4</v>
+        <v>0.48</v>
       </c>
       <c r="L2">
-        <v>0.45</v>
+        <v>0.495</v>
       </c>
     </row>
   </sheetData>
@@ -1241,7 +1262,7 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1258,7 +1279,7 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1275,7 +1296,7 @@
         <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1319,7 +1340,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1333,19 +1354,19 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1356,19 +1377,19 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
         <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1379,22 +1400,22 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1405,19 +1426,19 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G4" t="s">
         <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1428,19 +1449,19 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G5" t="s">
         <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1451,22 +1472,22 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1477,19 +1498,19 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G7" t="s">
         <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1500,22 +1521,22 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G8" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H8" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1532,10 +1553,10 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G9" t="s">
         <v>50</v>
@@ -1555,10 +1576,10 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G10" t="s">
         <v>50</v>
@@ -1578,10 +1599,10 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F11" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G11" t="s">
         <v>50</v>
@@ -1595,22 +1616,22 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G12" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H12" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1621,19 +1642,19 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G13" t="s">
         <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1644,22 +1665,22 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G14" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H14" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1676,10 +1697,10 @@
         <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G15" t="s">
         <v>50</v>
@@ -1699,10 +1720,10 @@
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G16" t="s">
         <v>50</v>
@@ -1722,10 +1743,10 @@
         <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F17" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G17" t="s">
         <v>50</v>
@@ -1739,22 +1760,22 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F18" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1765,19 +1786,19 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G19" t="s">
         <v>50</v>
       </c>
       <c r="H19" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1788,22 +1809,22 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G20" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H20" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1820,10 +1841,10 @@
         <v>32</v>
       </c>
       <c r="E21" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F21" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G21" t="s">
         <v>50</v>
@@ -1843,10 +1864,10 @@
         <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F22" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G22" t="s">
         <v>50</v>
@@ -1866,10 +1887,10 @@
         <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F23" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="G23" t="s">
         <v>50</v>
@@ -1883,22 +1904,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F24" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G24" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H24" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1909,19 +1930,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G25" t="s">
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1932,22 +1953,22 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E26" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G26" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H26" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1958,22 +1979,19 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F27" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="G27" t="s">
-        <v>108</v>
-      </c>
-      <c r="H27" t="s">
-        <v>110</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1984,22 +2002,19 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F28" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s">
-        <v>108</v>
-      </c>
-      <c r="H28" t="s">
-        <v>110</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2010,22 +2025,22 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="D29" t="s">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="F29" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G29" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H29" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2036,19 +2051,22 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="E30" t="s">
         <v>91</v>
       </c>
       <c r="F30" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="G30" t="s">
-        <v>50</v>
+        <v>114</v>
+      </c>
+      <c r="H30" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2059,22 +2077,19 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D31" t="s">
-        <v>75</v>
-      </c>
-      <c r="E31" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="F31" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G31" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="H31" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2085,22 +2100,22 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E32" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="F32" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G32" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H32" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2111,19 +2126,22 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D33" t="s">
-        <v>77</v>
+        <v>76</v>
+      </c>
+      <c r="E33" t="s">
+        <v>89</v>
       </c>
       <c r="F33" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G33" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="H33" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2134,22 +2152,22 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E34" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="F34" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G34" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H34" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2160,22 +2178,22 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E35" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F35" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G35" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H35" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2186,19 +2204,19 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="D36" t="s">
-        <v>80</v>
+        <v>41</v>
+      </c>
+      <c r="E36" t="s">
+        <v>96</v>
       </c>
       <c r="F36" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G36" t="s">
         <v>50</v>
-      </c>
-      <c r="H36" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2209,22 +2227,22 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E37" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="F37" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G37" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H37" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2235,22 +2253,22 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D38" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E38" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="F38" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G38" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H38" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2261,16 +2279,19 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" t="s">
-        <v>94</v>
+        <v>81</v>
+      </c>
+      <c r="D39" t="s">
+        <v>81</v>
       </c>
       <c r="F39" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G39" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="H39" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2281,16 +2302,22 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>18</v>
+        <v>82</v>
+      </c>
+      <c r="D40" t="s">
+        <v>82</v>
       </c>
       <c r="E40" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="F40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G40" t="s">
-        <v>49</v>
+        <v>114</v>
+      </c>
+      <c r="H40" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2301,16 +2328,22 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>22</v>
+        <v>83</v>
+      </c>
+      <c r="D41" t="s">
+        <v>83</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F41" t="s">
         <v>100</v>
       </c>
       <c r="G41" t="s">
-        <v>49</v>
+        <v>114</v>
+      </c>
+      <c r="H41" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2321,16 +2354,19 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>23</v>
-      </c>
-      <c r="E42" t="s">
-        <v>94</v>
+        <v>84</v>
+      </c>
+      <c r="D42" t="s">
+        <v>84</v>
       </c>
       <c r="F42" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G42" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="H42" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2341,16 +2377,22 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>85</v>
+      </c>
+      <c r="D43" t="s">
+        <v>85</v>
       </c>
       <c r="E43" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F43" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G43" t="s">
-        <v>49</v>
+        <v>114</v>
+      </c>
+      <c r="H43" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2361,16 +2403,22 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>25</v>
+        <v>86</v>
+      </c>
+      <c r="D44" t="s">
+        <v>86</v>
       </c>
       <c r="E44" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="F44" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G44" t="s">
-        <v>49</v>
+        <v>114</v>
+      </c>
+      <c r="H44" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2381,13 +2429,13 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E45" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F45" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G45" t="s">
         <v>49</v>
@@ -2401,13 +2449,13 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="E46" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F46" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G46" t="s">
         <v>49</v>
@@ -2421,13 +2469,13 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F47" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="G47" t="s">
         <v>49</v>
@@ -2441,13 +2489,13 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="E48" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F48" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G48" t="s">
         <v>49</v>
@@ -2461,13 +2509,13 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F49" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G49" t="s">
         <v>49</v>
@@ -2481,13 +2529,13 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E50" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F50" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="G50" t="s">
         <v>49</v>
@@ -2501,13 +2549,13 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E51" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F51" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="G51" t="s">
         <v>49</v>
@@ -2521,13 +2569,13 @@
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E52" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F52" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G52" t="s">
         <v>49</v>
@@ -2541,15 +2589,95 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
+        <v>31</v>
+      </c>
+      <c r="E53" t="s">
+        <v>100</v>
+      </c>
+      <c r="F53" t="s">
+        <v>95</v>
+      </c>
+      <c r="G53" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54" t="s">
+        <v>100</v>
+      </c>
+      <c r="F54" t="s">
+        <v>112</v>
+      </c>
+      <c r="G54" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" t="s">
+        <v>36</v>
+      </c>
+      <c r="E55" t="s">
+        <v>100</v>
+      </c>
+      <c r="F55" t="s">
+        <v>95</v>
+      </c>
+      <c r="G55" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>39</v>
+      </c>
+      <c r="E56" t="s">
+        <v>100</v>
+      </c>
+      <c r="F56" t="s">
+        <v>104</v>
+      </c>
+      <c r="G56" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
         <v>40</v>
       </c>
-      <c r="E53" t="s">
-        <v>94</v>
-      </c>
-      <c r="F53" t="s">
-        <v>107</v>
-      </c>
-      <c r="G53" t="s">
+      <c r="E57" t="s">
+        <v>100</v>
+      </c>
+      <c r="F57" t="s">
+        <v>113</v>
+      </c>
+      <c r="G57" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RDA maDMP JSON schema and related files; change model version and enhance dataset descriptions
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="106">
   <si>
     <t>rda model</t>
   </si>
@@ -49,7 +49,7 @@
     <t>f1</t>
   </si>
   <si>
-    <t>llama3.1:8b</t>
+    <t>gemma4:e4b</t>
   </si>
   <si>
     <t>sample</t>
@@ -232,15 +232,6 @@
     <t>dmp.dataset[2].type</t>
   </si>
   <si>
-    <t>dmp.dataset[3].dataset_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.dataset[3].dataset_id.type</t>
-  </si>
-  <si>
-    <t>dmp.dataset[3].type</t>
-  </si>
-  <si>
     <t>dmp.dmp_id.identifier</t>
   </si>
   <si>
@@ -262,46 +253,31 @@
     <t>dmp.project[0].description</t>
   </si>
   <si>
-    <t>dmp.project[0].funding[0].funder_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.project[0].funding[0].funder_id.type</t>
-  </si>
-  <si>
-    <t>dmp.project[0].funding[0].funding_status</t>
-  </si>
-  <si>
-    <t>dmp.related_identifier[0].identifier</t>
-  </si>
-  <si>
-    <t>dmp.related_identifier[0].relation_type</t>
-  </si>
-  <si>
-    <t>dmp.related_identifier[0].type</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>2026-10-19T00:00:00Z</t>
+    <t>dmp.project[0].start</t>
+  </si>
+  <si>
+    <t>2024-01-01T00:00:00Z</t>
   </si>
   <si>
     <t>no</t>
   </si>
   <si>
-    <t>Data related to each of our proposed experiments</t>
-  </si>
-  <si>
-    <t>dataset</t>
-  </si>
-  <si>
-    <t>Code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>Simulation code for controller development and testing</t>
-  </si>
-  <si>
-    <t>Software generated under the project</t>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>data related to each of our proposed experiments</t>
+  </si>
+  <si>
+    <t>raw data</t>
+  </si>
+  <si>
+    <t>code and results for all analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>code and results</t>
+  </si>
+  <si>
+    <t>simulation code for controller development and testing</t>
   </si>
   <si>
     <t>eng</t>
@@ -310,54 +286,42 @@
     <t>CPS 2015</t>
   </si>
   <si>
-    <t>The project aims to manage and disseminate data generated by the project.</t>
-  </si>
-  <si>
-    <t>planned</t>
-  </si>
-  <si>
-    <t>isPartOf</t>
+    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data. First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session. Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
+    <t>2024-01-01</t>
   </si>
   <si>
     <t>None</t>
   </si>
   <si>
-    <t>data related to each of our proposed experiments</t>
-  </si>
-  <si>
-    <t>code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>simulation code for controller development and testing</t>
+    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>servers at the Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+  </si>
+  <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+  </si>
+  <si>
+    <t>The code needed to generate all published results will be documented clearly.</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
+    <t>GNU Public License</t>
+  </si>
+  <si>
+    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
     <t>videos of the experiments</t>
   </si>
   <si>
-    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
-  </si>
-  <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
-  </si>
-  <si>
-    <t>The code needed to generate all published results will be documented clearly.</t>
-  </si>
-  <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
-    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
-  </si>
-  <si>
     <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
   </si>
   <si>
@@ -370,7 +334,7 @@
     <t>not in the reference</t>
   </si>
   <si>
-    <t>only 20% of the model's words are in the reference</t>
+    <t>different value</t>
   </si>
 </sst>
 </file>
@@ -774,25 +738,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="H2">
-        <v>0.512</v>
+        <v>0.594</v>
       </c>
       <c r="I2">
-        <v>0.48</v>
+        <v>0.28</v>
       </c>
       <c r="J2">
-        <v>0.495</v>
+        <v>0.381</v>
       </c>
     </row>
   </sheetData>
@@ -854,31 +818,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I2">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="J2">
-        <v>0.512</v>
+        <v>0.594</v>
       </c>
       <c r="K2">
-        <v>0.48</v>
+        <v>0.28</v>
       </c>
       <c r="L2">
-        <v>0.495</v>
+        <v>0.381</v>
       </c>
     </row>
   </sheetData>
@@ -973,7 +937,7 @@
         <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1092,7 +1056,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1194,7 +1158,7 @@
         <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1262,7 +1226,7 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1279,7 +1243,7 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1296,7 +1260,7 @@
         <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1340,7 +1304,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1383,13 +1347,13 @@
         <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G2" t="s">
         <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1405,17 +1369,14 @@
       <c r="D3" t="s">
         <v>58</v>
       </c>
-      <c r="E3" t="s">
-        <v>87</v>
-      </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G3" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1432,13 +1393,13 @@
         <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G4" t="s">
         <v>50</v>
       </c>
       <c r="H4" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1455,13 +1416,13 @@
         <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
         <v>50</v>
       </c>
       <c r="H5" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1478,16 +1439,16 @@
         <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H6" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1504,13 +1465,13 @@
         <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G7" t="s">
         <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1526,17 +1487,14 @@
       <c r="D8" t="s">
         <v>63</v>
       </c>
-      <c r="E8" t="s">
-        <v>87</v>
-      </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G8" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1553,10 +1511,10 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
         <v>50</v>
@@ -1576,13 +1534,16 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>50</v>
+        <v>102</v>
+      </c>
+      <c r="H10" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1599,10 +1560,10 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="G11" t="s">
         <v>50</v>
@@ -1622,16 +1583,16 @@
         <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H12" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1648,13 +1609,13 @@
         <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G13" t="s">
         <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1670,17 +1631,14 @@
       <c r="D14" t="s">
         <v>66</v>
       </c>
-      <c r="E14" t="s">
-        <v>87</v>
-      </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G14" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H14" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1697,10 +1655,10 @@
         <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
         <v>50</v>
@@ -1720,13 +1678,16 @@
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="F16" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G16" t="s">
-        <v>50</v>
+        <v>102</v>
+      </c>
+      <c r="H16" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1743,10 +1704,10 @@
         <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="G17" t="s">
         <v>50</v>
@@ -1766,16 +1727,16 @@
         <v>67</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H18" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1792,13 +1753,13 @@
         <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G19" t="s">
         <v>50</v>
       </c>
       <c r="H19" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1814,17 +1775,14 @@
       <c r="D20" t="s">
         <v>69</v>
       </c>
-      <c r="E20" t="s">
-        <v>87</v>
-      </c>
       <c r="F20" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G20" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H20" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1841,10 +1799,10 @@
         <v>32</v>
       </c>
       <c r="E21" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G21" t="s">
         <v>50</v>
@@ -1864,13 +1822,16 @@
         <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="F22" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G22" t="s">
-        <v>50</v>
+        <v>102</v>
+      </c>
+      <c r="H22" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1887,10 +1848,10 @@
         <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="G23" t="s">
         <v>50</v>
@@ -1910,16 +1871,16 @@
         <v>70</v>
       </c>
       <c r="E24" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F24" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G24" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H24" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1936,13 +1897,13 @@
         <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G25" t="s">
         <v>50</v>
       </c>
       <c r="H25" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1958,17 +1919,14 @@
       <c r="D26" t="s">
         <v>72</v>
       </c>
-      <c r="E26" t="s">
-        <v>87</v>
-      </c>
       <c r="F26" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G26" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H26" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1979,19 +1937,22 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="E27" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="F27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G27" t="s">
-        <v>50</v>
+        <v>102</v>
+      </c>
+      <c r="H27" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2002,19 +1963,22 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="D28" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="E28" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G28" t="s">
-        <v>50</v>
+        <v>102</v>
+      </c>
+      <c r="H28" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2025,22 +1989,22 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="D29" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="F29" t="s">
+        <v>91</v>
+      </c>
+      <c r="G29" t="s">
+        <v>102</v>
+      </c>
+      <c r="H29" t="s">
         <v>104</v>
-      </c>
-      <c r="G29" t="s">
-        <v>114</v>
-      </c>
-      <c r="H29" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2051,22 +2015,19 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="D30" t="s">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="E30" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F30" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="G30" t="s">
-        <v>114</v>
-      </c>
-      <c r="H30" t="s">
-        <v>116</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2077,19 +2038,22 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D31" t="s">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="E31" t="s">
+        <v>88</v>
       </c>
       <c r="F31" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G31" t="s">
-        <v>50</v>
+        <v>102</v>
       </c>
       <c r="H31" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2100,22 +2064,22 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D32" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F32" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G32" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H32" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2126,22 +2090,22 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E33" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F33" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G33" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H33" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2152,22 +2116,16 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
-      </c>
-      <c r="D34" t="s">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E34" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F34" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
-      </c>
-      <c r="H34" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2178,22 +2136,16 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>78</v>
-      </c>
-      <c r="D35" t="s">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F35" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="G35" t="s">
-        <v>114</v>
-      </c>
-      <c r="H35" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2204,19 +2156,16 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
-      </c>
-      <c r="D36" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F36" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="G36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2227,22 +2176,16 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
-      </c>
-      <c r="D37" t="s">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F37" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G37" t="s">
-        <v>114</v>
-      </c>
-      <c r="H37" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2253,22 +2196,16 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" t="s">
-        <v>80</v>
+        <v>23</v>
       </c>
       <c r="E38" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="F38" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G38" t="s">
-        <v>114</v>
-      </c>
-      <c r="H38" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2279,19 +2216,16 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
-      </c>
-      <c r="D39" t="s">
-        <v>81</v>
+        <v>24</v>
+      </c>
+      <c r="E39" t="s">
+        <v>91</v>
       </c>
       <c r="F39" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="G39" t="s">
-        <v>50</v>
-      </c>
-      <c r="H39" t="s">
-        <v>115</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2302,22 +2236,16 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
-      </c>
-      <c r="D40" t="s">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="E40" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F40" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G40" t="s">
-        <v>114</v>
-      </c>
-      <c r="H40" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2328,22 +2256,16 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>83</v>
-      </c>
-      <c r="D41" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="E41" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="F41" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G41" t="s">
-        <v>114</v>
-      </c>
-      <c r="H41" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2354,19 +2276,16 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
-      </c>
-      <c r="D42" t="s">
-        <v>84</v>
+        <v>29</v>
+      </c>
+      <c r="E42" t="s">
+        <v>91</v>
       </c>
       <c r="F42" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G42" t="s">
-        <v>50</v>
-      </c>
-      <c r="H42" t="s">
-        <v>115</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2377,22 +2296,16 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>85</v>
-      </c>
-      <c r="D43" t="s">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="E43" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="F43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G43" t="s">
-        <v>114</v>
-      </c>
-      <c r="H43" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2403,22 +2316,16 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>86</v>
-      </c>
-      <c r="D44" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="E44" t="s">
+        <v>91</v>
+      </c>
+      <c r="F44" t="s">
         <v>87</v>
       </c>
-      <c r="F44" t="s">
-        <v>100</v>
-      </c>
       <c r="G44" t="s">
-        <v>114</v>
-      </c>
-      <c r="H44" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2429,13 +2336,13 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E45" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F45" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="G45" t="s">
         <v>49</v>
@@ -2449,13 +2356,13 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E46" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F46" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="G46" t="s">
         <v>49</v>
@@ -2469,13 +2376,13 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="E47" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F47" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="G47" t="s">
         <v>49</v>
@@ -2489,13 +2396,13 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="E48" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F48" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="G48" t="s">
         <v>49</v>
@@ -2509,13 +2416,13 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="E49" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F49" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G49" t="s">
         <v>49</v>
@@ -2529,13 +2436,13 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E50" t="s">
+        <v>91</v>
+      </c>
+      <c r="F50" t="s">
         <v>100</v>
-      </c>
-      <c r="F50" t="s">
-        <v>109</v>
       </c>
       <c r="G50" t="s">
         <v>49</v>
@@ -2549,135 +2456,15 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="E51" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F51" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="G51" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52">
-        <v>3</v>
-      </c>
-      <c r="B52" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" t="s">
-        <v>100</v>
-      </c>
-      <c r="F52" t="s">
-        <v>111</v>
-      </c>
-      <c r="G52" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
-      <c r="A53">
-        <v>3</v>
-      </c>
-      <c r="B53" t="s">
-        <v>10</v>
-      </c>
-      <c r="C53" t="s">
-        <v>31</v>
-      </c>
-      <c r="E53" t="s">
-        <v>100</v>
-      </c>
-      <c r="F53" t="s">
-        <v>95</v>
-      </c>
-      <c r="G53" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
-      <c r="A54">
-        <v>3</v>
-      </c>
-      <c r="B54" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" t="s">
-        <v>35</v>
-      </c>
-      <c r="E54" t="s">
-        <v>100</v>
-      </c>
-      <c r="F54" t="s">
-        <v>112</v>
-      </c>
-      <c r="G54" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
-      <c r="A55">
-        <v>3</v>
-      </c>
-      <c r="B55" t="s">
-        <v>10</v>
-      </c>
-      <c r="C55" t="s">
-        <v>36</v>
-      </c>
-      <c r="E55" t="s">
-        <v>100</v>
-      </c>
-      <c r="F55" t="s">
-        <v>95</v>
-      </c>
-      <c r="G55" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56">
-        <v>3</v>
-      </c>
-      <c r="B56" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" t="s">
-        <v>39</v>
-      </c>
-      <c r="E56" t="s">
-        <v>100</v>
-      </c>
-      <c r="F56" t="s">
-        <v>104</v>
-      </c>
-      <c r="G56" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
-      <c r="A57">
-        <v>3</v>
-      </c>
-      <c r="B57" t="s">
-        <v>10</v>
-      </c>
-      <c r="C57" t="s">
-        <v>40</v>
-      </c>
-      <c r="E57" t="s">
-        <v>100</v>
-      </c>
-      <c r="F57" t="s">
-        <v>113</v>
-      </c>
-      <c r="G57" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new sample3 JSON files and update evaluation results and matrix images
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="132">
   <si>
     <t>rda model</t>
   </si>
@@ -166,15 +166,15 @@
     <t>Plan title &amp; description</t>
   </si>
   <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>Mismatch</t>
+  </si>
+  <si>
     <t>Missed</t>
   </si>
   <si>
-    <t>Correct</t>
-  </si>
-  <si>
-    <t>Mismatch</t>
-  </si>
-  <si>
     <t>model field</t>
   </si>
   <si>
@@ -211,7 +211,31 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[0].type</t>
+    <t>dmp.dataset[0].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].language</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dataset[1].dataset_id.identifier</t>
@@ -220,7 +244,28 @@
     <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[1].type</t>
+    <t>dmp.dataset[1].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[2].dataset_id.identifier</t>
@@ -229,7 +274,28 @@
     <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[2].type</t>
+    <t>dmp.dataset[2].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dmp_id.identifier</t>
@@ -253,43 +319,58 @@
     <t>dmp.project[0].description</t>
   </si>
   <si>
-    <t>dmp.project[0].start</t>
-  </si>
-  <si>
-    <t>2024-01-01T00:00:00Z</t>
+    <t>other</t>
+  </si>
+  <si>
+    <t>2026-10-19T00:00:00Z</t>
   </si>
   <si>
     <t>no</t>
   </si>
   <si>
+    <t>data related to each of our proposed experiments</t>
+  </si>
+  <si>
+    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>shared</t>
+  </si>
+  <si>
+    <t>Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>GNU Public License</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>eng</t>
+  </si>
+  <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+  </si>
+  <si>
+    <t>code and results for all analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
+    <t>simulation code for controller development and testing</t>
+  </si>
+  <si>
+    <t>These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
     <t>unknown</t>
   </si>
   <si>
-    <t>data related to each of our proposed experiments</t>
-  </si>
-  <si>
-    <t>raw data</t>
-  </si>
-  <si>
-    <t>code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>code and results</t>
-  </si>
-  <si>
-    <t>simulation code for controller development and testing</t>
-  </si>
-  <si>
-    <t>eng</t>
-  </si>
-  <si>
     <t>CPS 2015</t>
   </si>
   <si>
-    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data. First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session. Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>2024-01-01</t>
+    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
   </si>
   <si>
     <t>None</t>
@@ -304,27 +385,21 @@
     <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
   </si>
   <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+    <t>null</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
   </si>
   <si>
     <t>The code needed to generate all published results will be documented clearly.</t>
   </si>
   <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
     <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
     <t>videos of the experiments</t>
   </si>
   <si>
-    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
-  </si>
-  <si>
     <t>Hallucinated</t>
   </si>
   <si>
@@ -334,7 +409,10 @@
     <t>not in the reference</t>
   </si>
   <si>
-    <t>different value</t>
+    <t>only 57% of the model's words are in the reference</t>
+  </si>
+  <si>
+    <t>empty where the reference has a value</t>
   </si>
 </sst>
 </file>
@@ -738,25 +816,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="F2">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="G2">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H2">
-        <v>0.594</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="I2">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="J2">
-        <v>0.381</v>
+        <v>0.596</v>
       </c>
     </row>
   </sheetData>
@@ -818,31 +896,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="I2">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="J2">
-        <v>0.594</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="K2">
-        <v>0.28</v>
+        <v>0.64</v>
       </c>
       <c r="L2">
-        <v>0.381</v>
+        <v>0.596</v>
       </c>
     </row>
   </sheetData>
@@ -920,7 +998,7 @@
         <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -937,7 +1015,7 @@
         <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -954,7 +1032,7 @@
         <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -971,7 +1049,7 @@
         <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -988,7 +1066,7 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1022,7 +1100,7 @@
         <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1039,7 +1117,7 @@
         <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1056,7 +1134,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1073,7 +1151,7 @@
         <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1141,7 +1219,7 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1158,7 +1236,7 @@
         <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1175,7 +1253,7 @@
         <v>45</v>
       </c>
       <c r="E19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1192,7 +1270,7 @@
         <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1209,7 +1287,7 @@
         <v>46</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1226,7 +1304,7 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1243,7 +1321,7 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1260,7 +1338,7 @@
         <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1277,7 +1355,7 @@
         <v>48</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1294,7 +1372,7 @@
         <v>48</v>
       </c>
       <c r="E26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1304,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1347,13 +1425,13 @@
         <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1369,14 +1447,17 @@
       <c r="D3" t="s">
         <v>58</v>
       </c>
+      <c r="E3" t="s">
+        <v>100</v>
+      </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H3" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1393,13 +1474,13 @@
         <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1416,13 +1497,13 @@
         <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H5" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1439,16 +1520,16 @@
         <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H6" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1465,13 +1546,13 @@
         <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1487,14 +1568,17 @@
       <c r="D8" t="s">
         <v>63</v>
       </c>
+      <c r="E8" t="s">
+        <v>100</v>
+      </c>
       <c r="F8" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H8" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1511,13 +1595,13 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1534,16 +1618,13 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
-        <v>102</v>
-      </c>
-      <c r="H10" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1560,13 +1641,13 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1577,22 +1658,19 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
       <c r="G12" t="s">
-        <v>102</v>
-      </c>
-      <c r="H12" t="s">
-        <v>104</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1603,19 +1681,22 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="E13" t="s">
+        <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H13" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1626,19 +1707,19 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H14" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1649,19 +1730,19 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1672,22 +1753,19 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>102</v>
+        <v>49</v>
       </c>
       <c r="H16" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1698,19 +1776,22 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>127</v>
+      </c>
+      <c r="H17" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1721,22 +1802,22 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G18" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H18" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1747,19 +1828,22 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>69</v>
+      </c>
+      <c r="E19" t="s">
+        <v>109</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H19" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1770,19 +1854,19 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1793,19 +1877,22 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>127</v>
+      </c>
+      <c r="H21" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1816,22 +1903,19 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="E22" t="s">
-        <v>81</v>
-      </c>
-      <c r="F22" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="G22" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H22" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1842,19 +1926,19 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="F23" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="G23" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="H23" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1865,22 +1949,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="F24" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G24" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H24" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1891,19 +1975,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>26</v>
+      </c>
+      <c r="E25" t="s">
+        <v>102</v>
       </c>
       <c r="F25" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G25" t="s">
-        <v>50</v>
-      </c>
-      <c r="H25" t="s">
-        <v>103</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1914,19 +1998,19 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="D26" t="s">
-        <v>72</v>
+        <v>27</v>
+      </c>
+      <c r="E26" t="s">
+        <v>102</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="G26" t="s">
-        <v>50</v>
-      </c>
-      <c r="H26" t="s">
-        <v>103</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1937,22 +2021,19 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="D27" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="F27" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="G27" t="s">
-        <v>102</v>
-      </c>
-      <c r="H27" t="s">
-        <v>104</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1963,22 +2044,22 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="F28" t="s">
-        <v>91</v>
+        <v>121</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H28" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1995,16 +2076,16 @@
         <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="F29" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G29" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H29" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2015,19 +2096,19 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>76</v>
       </c>
       <c r="D30" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="F30" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G30" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="H30" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2038,22 +2119,22 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E31" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="F31" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="G31" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H31" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2064,22 +2145,19 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>77</v>
-      </c>
-      <c r="E32" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F32" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G32" t="s">
-        <v>102</v>
+        <v>49</v>
       </c>
       <c r="H32" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2090,22 +2168,22 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E33" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="F33" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="G33" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="H33" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2116,16 +2194,22 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>17</v>
+        <v>80</v>
+      </c>
+      <c r="D34" t="s">
+        <v>80</v>
       </c>
       <c r="E34" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="F34" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="G34" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H34" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2136,13 +2220,16 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>24</v>
+      </c>
+      <c r="D35" t="s">
+        <v>24</v>
       </c>
       <c r="E35" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="F35" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="G35" t="s">
         <v>49</v>
@@ -2156,16 +2243,19 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" t="s">
-        <v>91</v>
+        <v>81</v>
+      </c>
+      <c r="D36" t="s">
+        <v>81</v>
       </c>
       <c r="F36" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="G36" t="s">
         <v>49</v>
+      </c>
+      <c r="H36" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2176,16 +2266,22 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>22</v>
+        <v>82</v>
+      </c>
+      <c r="D37" t="s">
+        <v>82</v>
       </c>
       <c r="E37" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="F37" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="G37" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H37" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2198,14 +2294,17 @@
       <c r="C38" t="s">
         <v>23</v>
       </c>
-      <c r="E38" t="s">
-        <v>91</v>
+      <c r="D38" t="s">
+        <v>23</v>
       </c>
       <c r="F38" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="G38" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H38" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2216,16 +2315,19 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" t="s">
-        <v>91</v>
+        <v>83</v>
+      </c>
+      <c r="D39" t="s">
+        <v>83</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="G39" t="s">
         <v>49</v>
+      </c>
+      <c r="H39" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2236,16 +2338,22 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>25</v>
+        <v>84</v>
+      </c>
+      <c r="D40" t="s">
+        <v>84</v>
       </c>
       <c r="E40" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="F40" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="G40" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H40" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2256,13 +2364,16 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>27</v>
+        <v>32</v>
+      </c>
+      <c r="D41" t="s">
+        <v>32</v>
       </c>
       <c r="E41" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="F41" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G41" t="s">
         <v>49</v>
@@ -2276,13 +2387,16 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>29</v>
+        <v>33</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
       </c>
       <c r="E42" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="F42" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G42" t="s">
         <v>49</v>
@@ -2296,13 +2410,16 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="D43" t="s">
+        <v>34</v>
       </c>
       <c r="E43" t="s">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="F43" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="G43" t="s">
         <v>49</v>
@@ -2316,13 +2433,16 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>31</v>
+        <v>29</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
       </c>
       <c r="E44" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="F44" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="G44" t="s">
         <v>49</v>
@@ -2336,16 +2456,22 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>33</v>
+        <v>85</v>
+      </c>
+      <c r="D45" t="s">
+        <v>85</v>
       </c>
       <c r="E45" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="F45" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="G45" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H45" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2356,16 +2482,19 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>35</v>
-      </c>
-      <c r="E46" t="s">
-        <v>91</v>
+        <v>86</v>
+      </c>
+      <c r="D46" t="s">
+        <v>86</v>
       </c>
       <c r="F46" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="G46" t="s">
         <v>49</v>
+      </c>
+      <c r="H46" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2376,16 +2505,22 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>36</v>
+        <v>87</v>
+      </c>
+      <c r="D47" t="s">
+        <v>87</v>
       </c>
       <c r="E47" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="F47" t="s">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="G47" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="H47" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2396,76 +2531,542 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" t="s">
+        <v>88</v>
+      </c>
+      <c r="F48" t="s">
+        <v>118</v>
+      </c>
+      <c r="G48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H48" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>30</v>
+      </c>
+      <c r="D49" t="s">
+        <v>30</v>
+      </c>
+      <c r="E49" t="s">
+        <v>107</v>
+      </c>
+      <c r="F49" t="s">
+        <v>107</v>
+      </c>
+      <c r="G49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>89</v>
+      </c>
+      <c r="D50" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" t="s">
+        <v>108</v>
+      </c>
+      <c r="F50" t="s">
+        <v>118</v>
+      </c>
+      <c r="G50" t="s">
+        <v>127</v>
+      </c>
+      <c r="H50" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>31</v>
+      </c>
+      <c r="D51" t="s">
+        <v>31</v>
+      </c>
+      <c r="E51" t="s">
+        <v>109</v>
+      </c>
+      <c r="F51" t="s">
+        <v>109</v>
+      </c>
+      <c r="G51" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>90</v>
+      </c>
+      <c r="D52" t="s">
+        <v>90</v>
+      </c>
+      <c r="F52" t="s">
+        <v>118</v>
+      </c>
+      <c r="G52" t="s">
+        <v>49</v>
+      </c>
+      <c r="H52" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D53" t="s">
+        <v>91</v>
+      </c>
+      <c r="E53" t="s">
+        <v>100</v>
+      </c>
+      <c r="F53" t="s">
+        <v>118</v>
+      </c>
+      <c r="G53" t="s">
+        <v>127</v>
+      </c>
+      <c r="H53" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>92</v>
+      </c>
+      <c r="D54" t="s">
+        <v>92</v>
+      </c>
+      <c r="F54" t="s">
+        <v>118</v>
+      </c>
+      <c r="G54" t="s">
+        <v>49</v>
+      </c>
+      <c r="H54" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" t="s">
+        <v>93</v>
+      </c>
+      <c r="D55" t="s">
+        <v>93</v>
+      </c>
+      <c r="F55" t="s">
+        <v>118</v>
+      </c>
+      <c r="G55" t="s">
+        <v>49</v>
+      </c>
+      <c r="H55" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>94</v>
+      </c>
+      <c r="D56" t="s">
+        <v>94</v>
+      </c>
+      <c r="E56" t="s">
+        <v>100</v>
+      </c>
+      <c r="F56" t="s">
+        <v>118</v>
+      </c>
+      <c r="G56" t="s">
+        <v>127</v>
+      </c>
+      <c r="H56" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
+        <v>95</v>
+      </c>
+      <c r="D57" t="s">
+        <v>95</v>
+      </c>
+      <c r="E57" t="s">
+        <v>115</v>
+      </c>
+      <c r="F57" t="s">
+        <v>118</v>
+      </c>
+      <c r="G57" t="s">
+        <v>127</v>
+      </c>
+      <c r="H57" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58">
+        <v>3</v>
+      </c>
+      <c r="B58" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" t="s">
+        <v>96</v>
+      </c>
+      <c r="D58" t="s">
+        <v>96</v>
+      </c>
+      <c r="E58" t="s">
+        <v>109</v>
+      </c>
+      <c r="F58" t="s">
+        <v>118</v>
+      </c>
+      <c r="G58" t="s">
+        <v>127</v>
+      </c>
+      <c r="H58" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" t="s">
+        <v>97</v>
+      </c>
+      <c r="D59" t="s">
+        <v>97</v>
+      </c>
+      <c r="E59" t="s">
+        <v>101</v>
+      </c>
+      <c r="F59" t="s">
+        <v>118</v>
+      </c>
+      <c r="G59" t="s">
+        <v>127</v>
+      </c>
+      <c r="H59" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" t="s">
+        <v>41</v>
+      </c>
+      <c r="D60" t="s">
+        <v>41</v>
+      </c>
+      <c r="E60" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" t="s">
+        <v>116</v>
+      </c>
+      <c r="G60" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61">
+        <v>3</v>
+      </c>
+      <c r="B61" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" t="s">
+        <v>98</v>
+      </c>
+      <c r="D61" t="s">
+        <v>98</v>
+      </c>
+      <c r="F61" t="s">
+        <v>118</v>
+      </c>
+      <c r="G61" t="s">
+        <v>49</v>
+      </c>
+      <c r="H61" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62">
+        <v>3</v>
+      </c>
+      <c r="B62" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" t="s">
+        <v>99</v>
+      </c>
+      <c r="D62" t="s">
+        <v>99</v>
+      </c>
+      <c r="E62" t="s">
+        <v>117</v>
+      </c>
+      <c r="F62" t="s">
+        <v>118</v>
+      </c>
+      <c r="G62" t="s">
+        <v>127</v>
+      </c>
+      <c r="H62" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63">
+        <v>3</v>
+      </c>
+      <c r="B63" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" t="s">
+        <v>22</v>
+      </c>
+      <c r="E63" t="s">
+        <v>118</v>
+      </c>
+      <c r="F63" t="s">
+        <v>121</v>
+      </c>
+      <c r="G63" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64">
+        <v>3</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" t="s">
+        <v>23</v>
+      </c>
+      <c r="E64" t="s">
+        <v>118</v>
+      </c>
+      <c r="F64" t="s">
+        <v>110</v>
+      </c>
+      <c r="G64" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
+      <c r="A65">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
+        <v>25</v>
+      </c>
+      <c r="E65" t="s">
+        <v>118</v>
+      </c>
+      <c r="F65" t="s">
+        <v>124</v>
+      </c>
+      <c r="G65" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
+      <c r="A66">
+        <v>3</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>35</v>
+      </c>
+      <c r="E66" t="s">
+        <v>118</v>
+      </c>
+      <c r="F66" t="s">
+        <v>125</v>
+      </c>
+      <c r="G66" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
+      <c r="A67">
+        <v>3</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>36</v>
+      </c>
+      <c r="E67" t="s">
+        <v>118</v>
+      </c>
+      <c r="F67" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
+      <c r="A68">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" t="s">
         <v>37</v>
       </c>
-      <c r="E48" t="s">
-        <v>91</v>
-      </c>
-      <c r="F48" t="s">
-        <v>80</v>
-      </c>
-      <c r="G48" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49">
-        <v>3</v>
-      </c>
-      <c r="B49" t="s">
-        <v>10</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="E68" t="s">
+        <v>118</v>
+      </c>
+      <c r="F68" t="s">
+        <v>102</v>
+      </c>
+      <c r="G68" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
+      <c r="A69">
+        <v>3</v>
+      </c>
+      <c r="B69" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
         <v>38</v>
       </c>
-      <c r="E49" t="s">
-        <v>91</v>
-      </c>
-      <c r="F49" t="s">
-        <v>80</v>
-      </c>
-      <c r="G49" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50">
-        <v>3</v>
-      </c>
-      <c r="B50" t="s">
-        <v>10</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="E69" t="s">
+        <v>118</v>
+      </c>
+      <c r="F69" t="s">
+        <v>102</v>
+      </c>
+      <c r="G69" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
+      <c r="A70">
+        <v>3</v>
+      </c>
+      <c r="B70" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" t="s">
         <v>39</v>
       </c>
-      <c r="E50" t="s">
-        <v>91</v>
-      </c>
-      <c r="F50" t="s">
-        <v>100</v>
-      </c>
-      <c r="G50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51">
-        <v>3</v>
-      </c>
-      <c r="B51" t="s">
-        <v>10</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="E70" t="s">
+        <v>118</v>
+      </c>
+      <c r="F70" t="s">
+        <v>126</v>
+      </c>
+      <c r="G70" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
+      <c r="A71">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" t="s">
         <v>40</v>
       </c>
-      <c r="E51" t="s">
-        <v>91</v>
-      </c>
-      <c r="F51" t="s">
-        <v>101</v>
-      </c>
-      <c r="G51" t="s">
-        <v>49</v>
+      <c r="E71" t="s">
+        <v>118</v>
+      </c>
+      <c r="F71" t="s">
+        <v>117</v>
+      </c>
+      <c r="G71" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update evaluation results and add new sample JSON files for RDA evaluation
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="132">
   <si>
     <t>rda model</t>
   </si>
@@ -166,12 +166,15 @@
     <t>Plan title &amp; description</t>
   </si>
   <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>Mismatch</t>
+  </si>
+  <si>
     <t>Missed</t>
   </si>
   <si>
-    <t>Correct</t>
-  </si>
-  <si>
     <t>model field</t>
   </si>
   <si>
@@ -208,7 +211,31 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[0].type</t>
+    <t>dmp.dataset[0].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].language</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dataset[1].dataset_id.identifier</t>
@@ -217,7 +244,28 @@
     <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[1].type</t>
+    <t>dmp.dataset[1].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[2].dataset_id.identifier</t>
@@ -226,7 +274,28 @@
     <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
-    <t>dmp.dataset[2].type</t>
+    <t>dmp.dataset[2].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[2].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dmp_id.identifier</t>
@@ -253,7 +322,7 @@
     <t>other</t>
   </si>
   <si>
-    <t>2015-01-01T00:00:00Z</t>
+    <t>2026-10-19T00:00:00Z</t>
   </si>
   <si>
     <t>no</t>
@@ -262,25 +331,46 @@
     <t>data related to each of our proposed experiments</t>
   </si>
   <si>
-    <t>dataset</t>
+    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>shared</t>
+  </si>
+  <si>
+    <t>Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>GNU Public License</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>eng</t>
+  </si>
+  <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
   </si>
   <si>
     <t>code and results for all analyses completed on experimental data</t>
   </si>
   <si>
+    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
     <t>simulation code for controller development and testing</t>
   </si>
   <si>
+    <t>These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
     <t>unknown</t>
   </si>
   <si>
-    <t>eng</t>
-  </si>
-  <si>
     <t>CPS 2015</t>
   </si>
   <si>
-    <t>Data will be generated at each of our institutional sites. The PI at each institution will be responsible for following the data management guidelines described below, and for saving the data to the RIC servers. This process of transferring all data to a central location will be facilitated by our research project coordinator. Our data management guidelines will be reviewed at the kickoff meeting for the project, and revisited briefly at each of our quarterly meetings with the PIs.</t>
+    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
   </si>
   <si>
     <t>None</t>
@@ -295,27 +385,21 @@
     <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
   </si>
   <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+    <t>null</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
   </si>
   <si>
     <t>The code needed to generate all published results will be documented clearly.</t>
   </si>
   <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
     <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
   </si>
   <si>
     <t>videos of the experiments</t>
   </si>
   <si>
-    <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
-  </si>
-  <si>
     <t>Hallucinated</t>
   </si>
   <si>
@@ -323,6 +407,12 @@
   </si>
   <si>
     <t>not in the reference</t>
+  </si>
+  <si>
+    <t>only 57% of the model's words are in the reference</t>
+  </si>
+  <si>
+    <t>empty where the reference has a value</t>
   </si>
 </sst>
 </file>
@@ -726,25 +816,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="E2">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F2">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="H2">
-        <v>0.548</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="I2">
-        <v>0.4</v>
+        <v>0.64</v>
       </c>
       <c r="J2">
-        <v>0.463</v>
+        <v>0.596</v>
       </c>
     </row>
   </sheetData>
@@ -806,31 +896,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="J2">
-        <v>0.548</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="K2">
-        <v>0.4</v>
+        <v>0.64</v>
       </c>
       <c r="L2">
-        <v>0.463</v>
+        <v>0.596</v>
       </c>
     </row>
   </sheetData>
@@ -908,7 +998,7 @@
         <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -925,7 +1015,7 @@
         <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -942,7 +1032,7 @@
         <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -959,7 +1049,7 @@
         <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -976,7 +1066,7 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1010,7 +1100,7 @@
         <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1027,7 +1117,7 @@
         <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1044,7 +1134,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1061,7 +1151,7 @@
         <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1129,7 +1219,7 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1146,7 +1236,7 @@
         <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1163,7 +1253,7 @@
         <v>45</v>
       </c>
       <c r="E19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1180,7 +1270,7 @@
         <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1197,7 +1287,7 @@
         <v>46</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1214,7 +1304,7 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1231,7 +1321,7 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1248,7 +1338,7 @@
         <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1265,7 +1355,7 @@
         <v>48</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1282,7 +1372,7 @@
         <v>48</v>
       </c>
       <c r="E26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1292,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1306,19 +1396,19 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1329,19 +1419,19 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1352,22 +1442,22 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G3" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1378,19 +1468,19 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1401,19 +1491,19 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1424,22 +1514,22 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H6" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1450,19 +1540,19 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1473,22 +1563,22 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G8" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H8" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1505,13 +1595,13 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1528,13 +1618,13 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1551,13 +1641,13 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1568,22 +1658,19 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="G12" t="s">
-        <v>99</v>
-      </c>
-      <c r="H12" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1599,14 +1686,17 @@
       <c r="D13" t="s">
         <v>64</v>
       </c>
+      <c r="E13" t="s">
+        <v>105</v>
+      </c>
       <c r="F13" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1622,17 +1712,14 @@
       <c r="D14" t="s">
         <v>65</v>
       </c>
-      <c r="E14" t="s">
-        <v>77</v>
-      </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="H14" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1643,19 +1730,19 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1666,19 +1753,19 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="H16" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1689,19 +1776,22 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>127</v>
+      </c>
+      <c r="H17" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1712,22 +1802,22 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="F18" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G18" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H18" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1738,19 +1828,22 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="E19" t="s">
+        <v>109</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>50</v>
+        <v>127</v>
       </c>
       <c r="H19" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1761,22 +1854,19 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1787,19 +1877,22 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>127</v>
+      </c>
+      <c r="H21" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1810,19 +1903,19 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="E22" t="s">
-        <v>79</v>
-      </c>
-      <c r="F22" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="G22" t="s">
-        <v>50</v>
+        <v>127</v>
+      </c>
+      <c r="H22" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1833,19 +1926,19 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="F23" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="G23" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="H23" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1856,22 +1949,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="F24" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G24" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H24" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1882,19 +1975,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>26</v>
+      </c>
+      <c r="E25" t="s">
+        <v>102</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="G25" t="s">
-        <v>50</v>
-      </c>
-      <c r="H25" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1905,22 +1998,19 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E26" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="F26" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="G26" t="s">
-        <v>99</v>
-      </c>
-      <c r="H26" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1931,22 +2021,19 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="F27" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="G27" t="s">
-        <v>99</v>
-      </c>
-      <c r="H27" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1957,22 +2044,22 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="G28" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H28" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1983,22 +2070,22 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D29" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="F29" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="G29" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H29" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2009,19 +2096,19 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>76</v>
       </c>
       <c r="D30" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="F30" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="G30" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="H30" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2032,22 +2119,22 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E31" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="F31" t="s">
-        <v>88</v>
+        <v>122</v>
       </c>
       <c r="G31" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="H31" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2058,322 +2145,928 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>76</v>
-      </c>
-      <c r="E32" t="s">
+        <v>78</v>
+      </c>
+      <c r="F32" t="s">
+        <v>118</v>
+      </c>
+      <c r="G32" t="s">
+        <v>49</v>
+      </c>
+      <c r="H32" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" t="s">
+        <v>118</v>
+      </c>
+      <c r="G33" t="s">
+        <v>127</v>
+      </c>
+      <c r="H33" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" t="s">
+        <v>80</v>
+      </c>
+      <c r="E34" t="s">
+        <v>108</v>
+      </c>
+      <c r="F34" t="s">
+        <v>118</v>
+      </c>
+      <c r="G34" t="s">
+        <v>127</v>
+      </c>
+      <c r="H34" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36" t="s">
+        <v>81</v>
+      </c>
+      <c r="F36" t="s">
+        <v>118</v>
+      </c>
+      <c r="G36" t="s">
+        <v>49</v>
+      </c>
+      <c r="H36" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37" t="s">
+        <v>100</v>
+      </c>
+      <c r="F37" t="s">
+        <v>118</v>
+      </c>
+      <c r="G37" t="s">
+        <v>127</v>
+      </c>
+      <c r="H37" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38">
+        <v>3</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" t="s">
+        <v>110</v>
+      </c>
+      <c r="G38" t="s">
+        <v>127</v>
+      </c>
+      <c r="H38" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39">
+        <v>3</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" t="s">
+        <v>83</v>
+      </c>
+      <c r="D39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" t="s">
+        <v>118</v>
+      </c>
+      <c r="G39" t="s">
+        <v>49</v>
+      </c>
+      <c r="H39" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40">
+        <v>3</v>
+      </c>
+      <c r="B40" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" t="s">
+        <v>84</v>
+      </c>
+      <c r="D40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E40" t="s">
+        <v>100</v>
+      </c>
+      <c r="F40" t="s">
+        <v>118</v>
+      </c>
+      <c r="G40" t="s">
+        <v>127</v>
+      </c>
+      <c r="H40" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41">
+        <v>3</v>
+      </c>
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41" t="s">
+        <v>102</v>
+      </c>
+      <c r="G41" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42">
+        <v>3</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>33</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
+      </c>
+      <c r="E42" t="s">
+        <v>102</v>
+      </c>
+      <c r="F42" t="s">
+        <v>102</v>
+      </c>
+      <c r="G42" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43">
+        <v>3</v>
+      </c>
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" t="s">
+        <v>34</v>
+      </c>
+      <c r="D43" t="s">
+        <v>34</v>
+      </c>
+      <c r="E43" t="s">
+        <v>113</v>
+      </c>
+      <c r="F43" t="s">
+        <v>113</v>
+      </c>
+      <c r="G43" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44">
+        <v>3</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44" t="s">
+        <v>114</v>
+      </c>
+      <c r="F44" t="s">
+        <v>123</v>
+      </c>
+      <c r="G44" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45">
+        <v>3</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" t="s">
+        <v>85</v>
+      </c>
+      <c r="D45" t="s">
+        <v>85</v>
+      </c>
+      <c r="E45" t="s">
+        <v>105</v>
+      </c>
+      <c r="F45" t="s">
+        <v>118</v>
+      </c>
+      <c r="G45" t="s">
+        <v>127</v>
+      </c>
+      <c r="H45" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46">
+        <v>3</v>
+      </c>
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" t="s">
+        <v>86</v>
+      </c>
+      <c r="D46" t="s">
+        <v>86</v>
+      </c>
+      <c r="F46" t="s">
+        <v>118</v>
+      </c>
+      <c r="G46" t="s">
+        <v>49</v>
+      </c>
+      <c r="H46" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47">
+        <v>3</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" t="s">
         <v>87</v>
       </c>
-      <c r="F32" t="s">
+      <c r="D47" t="s">
+        <v>87</v>
+      </c>
+      <c r="E47" t="s">
+        <v>106</v>
+      </c>
+      <c r="F47" t="s">
+        <v>122</v>
+      </c>
+      <c r="G47" t="s">
+        <v>127</v>
+      </c>
+      <c r="H47" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
         <v>88</v>
       </c>
-      <c r="G32" t="s">
+      <c r="D48" t="s">
+        <v>88</v>
+      </c>
+      <c r="F48" t="s">
+        <v>118</v>
+      </c>
+      <c r="G48" t="s">
+        <v>49</v>
+      </c>
+      <c r="H48" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>30</v>
+      </c>
+      <c r="D49" t="s">
+        <v>30</v>
+      </c>
+      <c r="E49" t="s">
+        <v>107</v>
+      </c>
+      <c r="F49" t="s">
+        <v>107</v>
+      </c>
+      <c r="G49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>89</v>
+      </c>
+      <c r="D50" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" t="s">
+        <v>108</v>
+      </c>
+      <c r="F50" t="s">
+        <v>118</v>
+      </c>
+      <c r="G50" t="s">
+        <v>127</v>
+      </c>
+      <c r="H50" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>31</v>
+      </c>
+      <c r="D51" t="s">
+        <v>31</v>
+      </c>
+      <c r="E51" t="s">
+        <v>109</v>
+      </c>
+      <c r="F51" t="s">
+        <v>109</v>
+      </c>
+      <c r="G51" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>90</v>
+      </c>
+      <c r="D52" t="s">
+        <v>90</v>
+      </c>
+      <c r="F52" t="s">
+        <v>118</v>
+      </c>
+      <c r="G52" t="s">
+        <v>49</v>
+      </c>
+      <c r="H52" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D53" t="s">
+        <v>91</v>
+      </c>
+      <c r="E53" t="s">
+        <v>100</v>
+      </c>
+      <c r="F53" t="s">
+        <v>118</v>
+      </c>
+      <c r="G53" t="s">
+        <v>127</v>
+      </c>
+      <c r="H53" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>92</v>
+      </c>
+      <c r="D54" t="s">
+        <v>92</v>
+      </c>
+      <c r="F54" t="s">
+        <v>118</v>
+      </c>
+      <c r="G54" t="s">
+        <v>49</v>
+      </c>
+      <c r="H54" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" t="s">
+        <v>93</v>
+      </c>
+      <c r="D55" t="s">
+        <v>93</v>
+      </c>
+      <c r="F55" t="s">
+        <v>118</v>
+      </c>
+      <c r="G55" t="s">
+        <v>49</v>
+      </c>
+      <c r="H55" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>94</v>
+      </c>
+      <c r="D56" t="s">
+        <v>94</v>
+      </c>
+      <c r="E56" t="s">
+        <v>100</v>
+      </c>
+      <c r="F56" t="s">
+        <v>118</v>
+      </c>
+      <c r="G56" t="s">
+        <v>127</v>
+      </c>
+      <c r="H56" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" t="s">
+        <v>95</v>
+      </c>
+      <c r="D57" t="s">
+        <v>95</v>
+      </c>
+      <c r="E57" t="s">
+        <v>115</v>
+      </c>
+      <c r="F57" t="s">
+        <v>118</v>
+      </c>
+      <c r="G57" t="s">
+        <v>127</v>
+      </c>
+      <c r="H57" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58">
+        <v>3</v>
+      </c>
+      <c r="B58" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" t="s">
+        <v>96</v>
+      </c>
+      <c r="D58" t="s">
+        <v>96</v>
+      </c>
+      <c r="E58" t="s">
+        <v>109</v>
+      </c>
+      <c r="F58" t="s">
+        <v>118</v>
+      </c>
+      <c r="G58" t="s">
+        <v>127</v>
+      </c>
+      <c r="H58" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" t="s">
+        <v>97</v>
+      </c>
+      <c r="D59" t="s">
+        <v>97</v>
+      </c>
+      <c r="E59" t="s">
+        <v>101</v>
+      </c>
+      <c r="F59" t="s">
+        <v>118</v>
+      </c>
+      <c r="G59" t="s">
+        <v>127</v>
+      </c>
+      <c r="H59" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" t="s">
+        <v>41</v>
+      </c>
+      <c r="D60" t="s">
+        <v>41</v>
+      </c>
+      <c r="E60" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" t="s">
+        <v>116</v>
+      </c>
+      <c r="G60" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61">
+        <v>3</v>
+      </c>
+      <c r="B61" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" t="s">
+        <v>98</v>
+      </c>
+      <c r="D61" t="s">
+        <v>98</v>
+      </c>
+      <c r="F61" t="s">
+        <v>118</v>
+      </c>
+      <c r="G61" t="s">
+        <v>49</v>
+      </c>
+      <c r="H61" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62">
+        <v>3</v>
+      </c>
+      <c r="B62" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" t="s">
         <v>99</v>
       </c>
-      <c r="H32" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" t="s">
-        <v>88</v>
-      </c>
-      <c r="F33" t="s">
-        <v>89</v>
-      </c>
-      <c r="G33" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34">
-        <v>3</v>
-      </c>
-      <c r="B34" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" t="s">
-        <v>18</v>
-      </c>
-      <c r="E34" t="s">
-        <v>88</v>
-      </c>
-      <c r="F34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35">
-        <v>3</v>
-      </c>
-      <c r="B35" t="s">
-        <v>10</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="D62" t="s">
+        <v>99</v>
+      </c>
+      <c r="E62" t="s">
+        <v>117</v>
+      </c>
+      <c r="F62" t="s">
+        <v>118</v>
+      </c>
+      <c r="G62" t="s">
+        <v>127</v>
+      </c>
+      <c r="H62" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63">
+        <v>3</v>
+      </c>
+      <c r="B63" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" t="s">
         <v>22</v>
       </c>
-      <c r="E35" t="s">
-        <v>88</v>
-      </c>
-      <c r="F35" t="s">
-        <v>91</v>
-      </c>
-      <c r="G35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
-        <v>10</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="E63" t="s">
+        <v>118</v>
+      </c>
+      <c r="F63" t="s">
+        <v>121</v>
+      </c>
+      <c r="G63" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64">
+        <v>3</v>
+      </c>
+      <c r="B64" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" t="s">
         <v>23</v>
       </c>
-      <c r="E36" t="s">
-        <v>88</v>
-      </c>
-      <c r="F36" t="s">
-        <v>92</v>
-      </c>
-      <c r="G36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" t="s">
-        <v>24</v>
-      </c>
-      <c r="E37" t="s">
-        <v>88</v>
-      </c>
-      <c r="F37" t="s">
-        <v>85</v>
-      </c>
-      <c r="G37" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38">
-        <v>3</v>
-      </c>
-      <c r="B38" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="E64" t="s">
+        <v>118</v>
+      </c>
+      <c r="F64" t="s">
+        <v>110</v>
+      </c>
+      <c r="G64" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
+      <c r="A65">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
         <v>25</v>
       </c>
-      <c r="E38" t="s">
-        <v>88</v>
-      </c>
-      <c r="F38" t="s">
-        <v>93</v>
-      </c>
-      <c r="G38" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39">
-        <v>3</v>
-      </c>
-      <c r="B39" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" t="s">
-        <v>29</v>
-      </c>
-      <c r="E39" t="s">
-        <v>88</v>
-      </c>
-      <c r="F39" t="s">
-        <v>94</v>
-      </c>
-      <c r="G39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40">
-        <v>3</v>
-      </c>
-      <c r="B40" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" t="s">
-        <v>30</v>
-      </c>
-      <c r="E40" t="s">
-        <v>88</v>
-      </c>
-      <c r="F40" t="s">
-        <v>95</v>
-      </c>
-      <c r="G40" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41">
-        <v>3</v>
-      </c>
-      <c r="B41" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" t="s">
-        <v>31</v>
-      </c>
-      <c r="E41" t="s">
-        <v>88</v>
-      </c>
-      <c r="F41" t="s">
-        <v>85</v>
-      </c>
-      <c r="G41" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42">
-        <v>3</v>
-      </c>
-      <c r="B42" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="E65" t="s">
+        <v>118</v>
+      </c>
+      <c r="F65" t="s">
+        <v>124</v>
+      </c>
+      <c r="G65" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
+      <c r="A66">
+        <v>3</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
         <v>35</v>
       </c>
-      <c r="E42" t="s">
-        <v>88</v>
-      </c>
-      <c r="F42" t="s">
-        <v>96</v>
-      </c>
-      <c r="G42" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="B43" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="E66" t="s">
+        <v>118</v>
+      </c>
+      <c r="F66" t="s">
+        <v>125</v>
+      </c>
+      <c r="G66" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
+      <c r="A67">
+        <v>3</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
         <v>36</v>
       </c>
-      <c r="E43" t="s">
-        <v>88</v>
-      </c>
-      <c r="F43" t="s">
-        <v>85</v>
-      </c>
-      <c r="G43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44">
-        <v>3</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="E67" t="s">
+        <v>118</v>
+      </c>
+      <c r="F67" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
+      <c r="A68">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" t="s">
         <v>37</v>
       </c>
-      <c r="E44" t="s">
-        <v>88</v>
-      </c>
-      <c r="F44" t="s">
-        <v>79</v>
-      </c>
-      <c r="G44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45">
-        <v>3</v>
-      </c>
-      <c r="B45" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" t="s">
+      <c r="E68" t="s">
+        <v>118</v>
+      </c>
+      <c r="F68" t="s">
+        <v>102</v>
+      </c>
+      <c r="G68" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
+      <c r="A69">
+        <v>3</v>
+      </c>
+      <c r="B69" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
         <v>38</v>
       </c>
-      <c r="E45" t="s">
-        <v>88</v>
-      </c>
-      <c r="F45" t="s">
-        <v>79</v>
-      </c>
-      <c r="G45" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46">
-        <v>3</v>
-      </c>
-      <c r="B46" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="E69" t="s">
+        <v>118</v>
+      </c>
+      <c r="F69" t="s">
+        <v>102</v>
+      </c>
+      <c r="G69" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
+      <c r="A70">
+        <v>3</v>
+      </c>
+      <c r="B70" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" t="s">
         <v>39</v>
       </c>
-      <c r="E46" t="s">
-        <v>88</v>
-      </c>
-      <c r="F46" t="s">
-        <v>97</v>
-      </c>
-      <c r="G46" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47">
-        <v>3</v>
-      </c>
-      <c r="B47" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="E70" t="s">
+        <v>118</v>
+      </c>
+      <c r="F70" t="s">
+        <v>126</v>
+      </c>
+      <c r="G70" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
+      <c r="A71">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" t="s">
         <v>40</v>
       </c>
-      <c r="E47" t="s">
-        <v>88</v>
-      </c>
-      <c r="F47" t="s">
-        <v>98</v>
-      </c>
-      <c r="G47" t="s">
-        <v>49</v>
+      <c r="E71" t="s">
+        <v>118</v>
+      </c>
+      <c r="F71" t="s">
+        <v>117</v>
+      </c>
+      <c r="G71" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RDA model to llama3.3:70b and enhance DMP structure
- Changed RDA model from gemma4:e4b to llama3.3:70b in multiple JSON files and configuration.
- Updated prompt version from v10 to v12 and adjusted fingerprint accordingly.
- Expanded DMP JSON structure to include detailed dataset descriptions, distribution, and metadata requirements.
- Introduced a new output schema to enforce mandatory fields and improve model performance.
- Modified extraction and pipeline scripts to accommodate new schema and model changes.
- Enhanced tests to validate output schema and ensure correct fingerprinting behavior.
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="166">
   <si>
     <t>rda model</t>
   </si>
@@ -49,7 +49,7 @@
     <t>f1</t>
   </si>
   <si>
-    <t>gemma4:e4b</t>
+    <t>llama3.3:70b</t>
   </si>
   <si>
     <t>sample</t>
@@ -190,19 +190,37 @@
     <t>reason</t>
   </si>
   <si>
+    <t>dmp.created</t>
+  </si>
+  <si>
+    <t>dmp.modified</t>
+  </si>
+  <si>
+    <t>dmp.language</t>
+  </si>
+  <si>
+    <t>dmp.ethical_issues_exist</t>
+  </si>
+  <si>
+    <t>dmp.dmp_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dmp_id.type</t>
+  </si>
+  <si>
+    <t>dmp.contact.name</t>
+  </si>
+  <si>
+    <t>dmp.contact.mbox</t>
+  </si>
+  <si>
     <t>dmp.contact.contact_id[0].identifier</t>
   </si>
   <si>
     <t>dmp.contact.contact_id[0].type</t>
   </si>
   <si>
-    <t>dmp.contact.mbox</t>
-  </si>
-  <si>
-    <t>dmp.contact.name</t>
-  </si>
-  <si>
-    <t>dmp.created</t>
+    <t>dmp.dataset[0].type</t>
   </si>
   <si>
     <t>dmp.dataset[0].dataset_id.identifier</t>
@@ -211,19 +229,40 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
+    <t>dmp.dataset[0].distribution[0].title</t>
+  </si>
+  <si>
     <t>dmp.dataset[0].distribution[0].data_access</t>
   </si>
   <si>
-    <t>dmp.dataset[0].distribution[0].title</t>
+    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
   </si>
   <si>
     <t>dmp.dataset[0].distribution[0].host.url</t>
   </si>
   <si>
-    <t>dmp.dataset[0].distribution[0].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[0].license[0].start_date</t>
+    <t>dmp.dataset[0].distribution[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dataset[0].metadata[0].language</t>
@@ -235,7 +274,7 @@
     <t>dmp.dataset[0].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
-    <t>dmp.dataset[0].metadata[0].description</t>
+    <t>dmp.dataset[1].type</t>
   </si>
   <si>
     <t>dmp.dataset[1].dataset_id.identifier</t>
@@ -244,10 +283,16 @@
     <t>dmp.dataset[1].dataset_id.type</t>
   </si>
   <si>
+    <t>dmp.dataset[1].distribution[0].title</t>
+  </si>
+  <si>
     <t>dmp.dataset[1].distribution[0].data_access</t>
   </si>
   <si>
-    <t>dmp.dataset[1].distribution[0].title</t>
+    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
   </si>
   <si>
     <t>dmp.dataset[1].distribution[0].host.title</t>
@@ -256,10 +301,22 @@
     <t>dmp.dataset[1].distribution[0].host.url</t>
   </si>
   <si>
-    <t>dmp.dataset[1].distribution[0].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[0].license[0].start_date</t>
+    <t>dmp.dataset[1].distribution[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[1].distribution[1].host.url</t>
   </si>
   <si>
     <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
@@ -268,16 +325,22 @@
     <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
+    <t>dmp.dataset[2].type</t>
+  </si>
+  <si>
     <t>dmp.dataset[2].dataset_id.identifier</t>
   </si>
   <si>
     <t>dmp.dataset[2].dataset_id.type</t>
   </si>
   <si>
+    <t>dmp.dataset[2].distribution[0].title</t>
+  </si>
+  <si>
     <t>dmp.dataset[2].distribution[0].data_access</t>
   </si>
   <si>
-    <t>dmp.dataset[2].distribution[0].title</t>
+    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
   </si>
   <si>
     <t>dmp.dataset[2].distribution[0].host.title</t>
@@ -286,7 +349,7 @@
     <t>dmp.dataset[2].distribution[0].host.url</t>
   </si>
   <si>
-    <t>dmp.dataset[2].distribution[0].license[0].start_date</t>
+    <t>dmp.dataset[2].metadata[0].description</t>
   </si>
   <si>
     <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].identifier</t>
@@ -295,22 +358,40 @@
     <t>dmp.dataset[2].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
-    <t>dmp.dataset[2].metadata[0].description</t>
-  </si>
-  <si>
-    <t>dmp.dmp_id.identifier</t>
-  </si>
-  <si>
-    <t>dmp.dmp_id.type</t>
-  </si>
-  <si>
-    <t>dmp.ethical_issues_exist</t>
-  </si>
-  <si>
-    <t>dmp.language</t>
-  </si>
-  <si>
-    <t>dmp.modified</t>
+    <t>dmp.dataset[3].type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].dataset_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].dataset_id.type</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].distribution[0].host.url</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].metadata[0].description</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].metadata[0].metadata_standard_id[0].identifier</t>
+  </si>
+  <si>
+    <t>dmp.dataset[3].metadata[0].metadata_standard_id[0].type</t>
   </si>
   <si>
     <t>dmp.project[0].title</t>
@@ -319,100 +400,121 @@
     <t>dmp.project[0].description</t>
   </si>
   <si>
+    <t>dmp.project[0].funding[0].funder_id.identifier</t>
+  </si>
+  <si>
+    <t>dmp.project[0].funding[0].funder_id.type</t>
+  </si>
+  <si>
+    <t>dmp.project[0].funding[0].funding_status</t>
+  </si>
+  <si>
+    <t>CPS 2015</t>
+  </si>
+  <si>
+    <t>2026-10-19T00:00:00Z</t>
+  </si>
+  <si>
+    <t>eng</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
     <t>other</t>
   </si>
   <si>
-    <t>2026-10-19T00:00:00Z</t>
+    <t>data related to each of our proposed experiments</t>
+  </si>
+  <si>
+    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>dataset</t>
   </si>
   <si>
     <t>no</t>
   </si>
   <si>
-    <t>data related to each of our proposed experiments</t>
-  </si>
-  <si>
-    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
     <t>shared</t>
   </si>
   <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>project's website</t>
+  </si>
+  <si>
     <t>Rehabilitation Institute of Chicago</t>
   </si>
   <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+  </si>
+  <si>
+    <t>code and results for all analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+  </si>
+  <si>
+    <t>simulation code for controller development and testing</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
     <t>GNU Public License</t>
   </si>
   <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>eng</t>
-  </si>
-  <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
-  </si>
-  <si>
-    <t>code and results for all analyses completed on experimental data</t>
-  </si>
-  <si>
-    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts. The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>simulation code for controller development and testing</t>
-  </si>
-  <si>
-    <t>These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>unknown</t>
-  </si>
-  <si>
-    <t>CPS 2015</t>
+    <t>labs' websites</t>
+  </si>
+  <si>
+    <t>select videos of the experiments</t>
+  </si>
+  <si>
+    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
+  </si>
+  <si>
+    <t>The Data Management Plan should clearly articulate how the PI and co-PIs plan to manage and disseminate data generated by the project.</t>
+  </si>
+  <si>
+    <t>planned</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>servers at the Rehabilitation Institute of Chicago</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+  </si>
+  <si>
+    <t>videos of the experiments</t>
+  </si>
+  <si>
+    <t>The code needed to generate all published results will be documented clearly.</t>
   </si>
   <si>
     <t>We will manage all scientific and technical content generated from this proposal. Our products will include 3 broad types of data.</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
-  </si>
-  <si>
-    <t>null</t>
-  </si>
-  <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>The code needed to generate all published results will be documented clearly.</t>
-  </si>
-  <si>
-    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
-  </si>
-  <si>
-    <t>videos of the experiments</t>
-  </si>
-  <si>
     <t>Hallucinated</t>
   </si>
   <si>
+    <t>not in the reference</t>
+  </si>
+  <si>
     <t>both empty</t>
   </si>
   <si>
-    <t>not in the reference</t>
-  </si>
-  <si>
-    <t>only 57% of the model's words are in the reference</t>
-  </si>
-  <si>
-    <t>empty where the reference has a value</t>
+    <t>only 0% of the model's words are in the reference</t>
   </si>
 </sst>
 </file>
@@ -816,25 +918,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="E2">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="F2">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="G2">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>0.5570000000000001</v>
+        <v>0.542</v>
       </c>
       <c r="I2">
-        <v>0.64</v>
+        <v>0.88</v>
       </c>
       <c r="J2">
-        <v>0.596</v>
+        <v>0.671</v>
       </c>
     </row>
   </sheetData>
@@ -896,31 +998,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="I2">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="J2">
-        <v>0.5570000000000001</v>
+        <v>0.542</v>
       </c>
       <c r="K2">
-        <v>0.64</v>
+        <v>0.88</v>
       </c>
       <c r="L2">
-        <v>0.596</v>
+        <v>0.671</v>
       </c>
     </row>
   </sheetData>
@@ -981,7 +1083,7 @@
         <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1049,7 +1151,7 @@
         <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1066,7 +1168,7 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1270,7 +1372,7 @@
         <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1287,7 +1389,7 @@
         <v>46</v>
       </c>
       <c r="E21" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1304,7 +1406,7 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1321,7 +1423,7 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1338,7 +1440,7 @@
         <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1382,7 +1484,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1419,19 +1521,19 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>41</v>
+      </c>
+      <c r="E2" t="s">
+        <v>130</v>
       </c>
       <c r="F2" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="G2" t="s">
         <v>49</v>
-      </c>
-      <c r="H2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1442,22 +1544,22 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>131</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G3" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H3" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1468,19 +1570,22 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>58</v>
+      </c>
+      <c r="E4" t="s">
+        <v>131</v>
       </c>
       <c r="F4" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G4" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H4" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1491,19 +1596,22 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>59</v>
+      </c>
+      <c r="E5" t="s">
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G5" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H5" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1514,22 +1622,22 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G6" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H6" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1540,19 +1648,19 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1563,22 +1671,22 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>100</v>
+        <v>134</v>
       </c>
       <c r="F8" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G8" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H8" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1589,19 +1697,19 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" t="s">
-        <v>102</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G9" t="s">
         <v>49</v>
+      </c>
+      <c r="H9" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1612,19 +1720,19 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G10" t="s">
         <v>49</v>
+      </c>
+      <c r="H10" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1635,19 +1743,19 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
       <c r="G11" t="s">
         <v>49</v>
+      </c>
+      <c r="H11" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1658,19 +1766,22 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="F12" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="G12" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H12" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1681,22 +1792,19 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="F13" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="G13" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1707,19 +1815,19 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>136</v>
       </c>
       <c r="F14" t="s">
-        <v>118</v>
+        <v>155</v>
       </c>
       <c r="G14" t="s">
         <v>49</v>
-      </c>
-      <c r="H14" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1730,19 +1838,22 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="F15" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="G15" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H15" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1753,19 +1864,19 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>138</v>
       </c>
       <c r="F16" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="G16" t="s">
         <v>49</v>
-      </c>
-      <c r="H16" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1776,22 +1887,19 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="F17" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="G17" t="s">
-        <v>127</v>
-      </c>
-      <c r="H17" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1807,17 +1915,14 @@
       <c r="D18" t="s">
         <v>68</v>
       </c>
-      <c r="E18" t="s">
-        <v>108</v>
-      </c>
       <c r="F18" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G18" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H18" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1834,16 +1939,16 @@
         <v>69</v>
       </c>
       <c r="E19" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="F19" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G19" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H19" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1860,13 +1965,13 @@
         <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1883,16 +1988,16 @@
         <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="F21" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G21" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H21" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1908,14 +2013,14 @@
       <c r="D22" t="s">
         <v>72</v>
       </c>
-      <c r="E22" t="s">
-        <v>110</v>
+      <c r="F22" t="s">
+        <v>154</v>
       </c>
       <c r="G22" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H22" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1931,14 +2036,17 @@
       <c r="D23" t="s">
         <v>73</v>
       </c>
+      <c r="E23" t="s">
+        <v>140</v>
+      </c>
       <c r="F23" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G23" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H23" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1949,22 +2057,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="F24" t="s">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="G24" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H24" t="s">
-        <v>129</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1975,19 +2083,19 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="D25" t="s">
-        <v>26</v>
-      </c>
-      <c r="E25" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="F25" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G25" t="s">
         <v>49</v>
+      </c>
+      <c r="H25" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1998,19 +2106,19 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="F26" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G26" t="s">
         <v>49</v>
+      </c>
+      <c r="H26" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2021,19 +2129,22 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="E27" t="s">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="F27" t="s">
-        <v>111</v>
+        <v>154</v>
       </c>
       <c r="G27" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H27" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2044,22 +2155,19 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>154</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2070,22 +2178,22 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D29" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="F29" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G29" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H29" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2096,19 +2204,22 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>79</v>
+      </c>
+      <c r="E30" t="s">
+        <v>142</v>
       </c>
       <c r="F30" t="s">
-        <v>118</v>
+        <v>157</v>
       </c>
       <c r="G30" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H30" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2119,22 +2230,19 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D31" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="F31" t="s">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="G31" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H31" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2145,19 +2253,19 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
-      </c>
-      <c r="F32" t="s">
-        <v>118</v>
+        <v>81</v>
+      </c>
+      <c r="E32" t="s">
+        <v>143</v>
       </c>
       <c r="G32" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H32" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2168,22 +2276,22 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D33" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E33" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="F33" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G33" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H33" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2194,22 +2302,19 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D34" t="s">
-        <v>80</v>
-      </c>
-      <c r="E34" t="s">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="F34" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G34" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H34" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2220,19 +2325,22 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="D35" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="E35" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="F35" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="G35" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H35" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2243,19 +2351,19 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="D36" t="s">
-        <v>81</v>
+        <v>28</v>
+      </c>
+      <c r="E36" t="s">
+        <v>144</v>
       </c>
       <c r="F36" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="G36" t="s">
         <v>49</v>
-      </c>
-      <c r="H36" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2266,22 +2374,19 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="F37" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="G37" t="s">
-        <v>127</v>
-      </c>
-      <c r="H37" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2292,19 +2397,22 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="D38" t="s">
-        <v>23</v>
+        <v>85</v>
+      </c>
+      <c r="E38" t="s">
+        <v>137</v>
       </c>
       <c r="F38" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="G38" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H38" t="s">
-        <v>131</v>
+        <v>163</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2315,19 +2423,19 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="D39" t="s">
-        <v>83</v>
+        <v>26</v>
+      </c>
+      <c r="E39" t="s">
+        <v>138</v>
       </c>
       <c r="F39" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="G39" t="s">
         <v>49</v>
-      </c>
-      <c r="H39" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2338,22 +2446,19 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="D40" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="E40" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F40" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="G40" t="s">
-        <v>127</v>
-      </c>
-      <c r="H40" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2364,19 +2469,19 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="D41" t="s">
-        <v>32</v>
-      </c>
-      <c r="E41" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F41" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G41" t="s">
         <v>49</v>
+      </c>
+      <c r="H41" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2387,19 +2492,22 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="D42" t="s">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="E42" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="F42" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="G42" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H42" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2410,19 +2518,19 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="D43" t="s">
-        <v>34</v>
-      </c>
-      <c r="E43" t="s">
-        <v>113</v>
+        <v>88</v>
       </c>
       <c r="F43" t="s">
-        <v>113</v>
+        <v>154</v>
       </c>
       <c r="G43" t="s">
         <v>49</v>
+      </c>
+      <c r="H43" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2433,19 +2541,22 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="D44" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="E44" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="F44" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="G44" t="s">
-        <v>49</v>
+        <v>162</v>
+      </c>
+      <c r="H44" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2456,22 +2567,19 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D45" t="s">
-        <v>85</v>
-      </c>
-      <c r="E45" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="F45" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G45" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H45" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2482,19 +2590,22 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D46" t="s">
-        <v>86</v>
+        <v>91</v>
+      </c>
+      <c r="E46" t="s">
+        <v>140</v>
       </c>
       <c r="F46" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G46" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H46" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2505,22 +2616,22 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D47" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="E47" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="F47" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="G47" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H47" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2531,19 +2642,19 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D48" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F48" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G48" t="s">
         <v>49</v>
       </c>
       <c r="H48" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2554,19 +2665,19 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="D49" t="s">
-        <v>30</v>
-      </c>
-      <c r="E49" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="F49" t="s">
-        <v>107</v>
+        <v>154</v>
       </c>
       <c r="G49" t="s">
         <v>49</v>
+      </c>
+      <c r="H49" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2577,22 +2688,22 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D50" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E50" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G50" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H50" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2603,19 +2714,19 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="D51" t="s">
-        <v>31</v>
-      </c>
-      <c r="E51" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="F51" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="G51" t="s">
         <v>49</v>
+      </c>
+      <c r="H51" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2626,19 +2737,22 @@
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D52" t="s">
-        <v>90</v>
+        <v>97</v>
+      </c>
+      <c r="E52" t="s">
+        <v>140</v>
       </c>
       <c r="F52" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G52" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H52" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2649,22 +2763,22 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D53" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="E53" t="s">
-        <v>100</v>
+        <v>142</v>
       </c>
       <c r="F53" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G53" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H53" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2675,19 +2789,19 @@
         <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D54" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="F54" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G54" t="s">
         <v>49</v>
       </c>
       <c r="H54" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2698,19 +2812,19 @@
         <v>10</v>
       </c>
       <c r="C55" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="D55" t="s">
-        <v>93</v>
+        <v>23</v>
+      </c>
+      <c r="E55" t="s">
+        <v>143</v>
       </c>
       <c r="F55" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="G55" t="s">
         <v>49</v>
-      </c>
-      <c r="H55" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2721,22 +2835,19 @@
         <v>10</v>
       </c>
       <c r="C56" t="s">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="D56" t="s">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="F56" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="G56" t="s">
-        <v>127</v>
-      </c>
-      <c r="H56" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2747,22 +2858,19 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D57" t="s">
-        <v>95</v>
-      </c>
-      <c r="E57" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="F57" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G57" t="s">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="H57" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2773,22 +2881,22 @@
         <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D58" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E58" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="F58" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G58" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H58" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2799,22 +2907,19 @@
         <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="D59" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E59" t="s">
-        <v>101</v>
+        <v>146</v>
       </c>
       <c r="F59" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="G59" t="s">
-        <v>127</v>
-      </c>
-      <c r="H59" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2825,16 +2930,16 @@
         <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D60" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="E60" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="F60" t="s">
-        <v>116</v>
+        <v>147</v>
       </c>
       <c r="G60" t="s">
         <v>49</v>
@@ -2848,19 +2953,22 @@
         <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D61" t="s">
-        <v>98</v>
+        <v>102</v>
+      </c>
+      <c r="E61" t="s">
+        <v>137</v>
       </c>
       <c r="F61" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="G61" t="s">
-        <v>49</v>
+        <v>162</v>
       </c>
       <c r="H61" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2871,22 +2979,19 @@
         <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="D62" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="E62" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="F62" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="G62" t="s">
-        <v>127</v>
-      </c>
-      <c r="H62" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2897,16 +3002,19 @@
         <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>22</v>
+        <v>33</v>
+      </c>
+      <c r="D63" t="s">
+        <v>33</v>
       </c>
       <c r="E63" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="F63" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="G63" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2917,155 +3025,888 @@
         <v>10</v>
       </c>
       <c r="C64" t="s">
-        <v>23</v>
-      </c>
-      <c r="E64" t="s">
+        <v>103</v>
+      </c>
+      <c r="D64" t="s">
+        <v>103</v>
+      </c>
+      <c r="F64" t="s">
+        <v>154</v>
+      </c>
+      <c r="G64" t="s">
+        <v>49</v>
+      </c>
+      <c r="H64" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
+        <v>104</v>
+      </c>
+      <c r="D65" t="s">
+        <v>104</v>
+      </c>
+      <c r="E65" t="s">
+        <v>134</v>
+      </c>
+      <c r="F65" t="s">
+        <v>154</v>
+      </c>
+      <c r="G65" t="s">
+        <v>162</v>
+      </c>
+      <c r="H65" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66">
+        <v>3</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>105</v>
+      </c>
+      <c r="D66" t="s">
+        <v>105</v>
+      </c>
+      <c r="F66" t="s">
+        <v>154</v>
+      </c>
+      <c r="G66" t="s">
+        <v>49</v>
+      </c>
+      <c r="H66" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67">
+        <v>3</v>
+      </c>
+      <c r="B67" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" t="s">
+        <v>106</v>
+      </c>
+      <c r="D67" t="s">
+        <v>106</v>
+      </c>
+      <c r="E67" t="s">
+        <v>139</v>
+      </c>
+      <c r="F67" t="s">
+        <v>154</v>
+      </c>
+      <c r="G67" t="s">
+        <v>162</v>
+      </c>
+      <c r="H67" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" t="s">
+        <v>30</v>
+      </c>
+      <c r="D68" t="s">
+        <v>30</v>
+      </c>
+      <c r="E68" t="s">
+        <v>148</v>
+      </c>
+      <c r="F68" t="s">
+        <v>148</v>
+      </c>
+      <c r="G68" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69">
+        <v>3</v>
+      </c>
+      <c r="B69" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
+        <v>107</v>
+      </c>
+      <c r="D69" t="s">
+        <v>107</v>
+      </c>
+      <c r="E69" t="s">
+        <v>140</v>
+      </c>
+      <c r="F69" t="s">
+        <v>154</v>
+      </c>
+      <c r="G69" t="s">
+        <v>162</v>
+      </c>
+      <c r="H69" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70">
+        <v>3</v>
+      </c>
+      <c r="B70" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" t="s">
+        <v>108</v>
+      </c>
+      <c r="D70" t="s">
+        <v>108</v>
+      </c>
+      <c r="E70" t="s">
+        <v>149</v>
+      </c>
+      <c r="F70" t="s">
+        <v>157</v>
+      </c>
+      <c r="G70" t="s">
+        <v>162</v>
+      </c>
+      <c r="H70" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" t="s">
+        <v>109</v>
+      </c>
+      <c r="D71" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" t="s">
+        <v>154</v>
+      </c>
+      <c r="G71" t="s">
+        <v>49</v>
+      </c>
+      <c r="H71" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72">
+        <v>3</v>
+      </c>
+      <c r="B72" t="s">
+        <v>10</v>
+      </c>
+      <c r="C72" t="s">
+        <v>110</v>
+      </c>
+      <c r="D72" t="s">
+        <v>110</v>
+      </c>
+      <c r="E72" t="s">
+        <v>143</v>
+      </c>
+      <c r="F72" t="s">
+        <v>154</v>
+      </c>
+      <c r="G72" t="s">
+        <v>162</v>
+      </c>
+      <c r="H72" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73">
+        <v>3</v>
+      </c>
+      <c r="B73" t="s">
+        <v>10</v>
+      </c>
+      <c r="C73" t="s">
+        <v>31</v>
+      </c>
+      <c r="D73" t="s">
+        <v>31</v>
+      </c>
+      <c r="E73" t="s">
+        <v>132</v>
+      </c>
+      <c r="F73" t="s">
+        <v>132</v>
+      </c>
+      <c r="G73" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74">
+        <v>3</v>
+      </c>
+      <c r="B74" t="s">
+        <v>10</v>
+      </c>
+      <c r="C74" t="s">
+        <v>111</v>
+      </c>
+      <c r="D74" t="s">
+        <v>111</v>
+      </c>
+      <c r="F74" t="s">
+        <v>154</v>
+      </c>
+      <c r="G74" t="s">
+        <v>49</v>
+      </c>
+      <c r="H74" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75">
+        <v>3</v>
+      </c>
+      <c r="B75" t="s">
+        <v>10</v>
+      </c>
+      <c r="C75" t="s">
+        <v>112</v>
+      </c>
+      <c r="D75" t="s">
+        <v>112</v>
+      </c>
+      <c r="E75" t="s">
+        <v>134</v>
+      </c>
+      <c r="F75" t="s">
+        <v>154</v>
+      </c>
+      <c r="G75" t="s">
+        <v>162</v>
+      </c>
+      <c r="H75" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76">
+        <v>3</v>
+      </c>
+      <c r="B76" t="s">
+        <v>10</v>
+      </c>
+      <c r="C76" t="s">
+        <v>39</v>
+      </c>
+      <c r="D76" t="s">
+        <v>39</v>
+      </c>
+      <c r="E76" t="s">
+        <v>150</v>
+      </c>
+      <c r="F76" t="s">
+        <v>159</v>
+      </c>
+      <c r="G76" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77">
+        <v>3</v>
+      </c>
+      <c r="B77" t="s">
+        <v>10</v>
+      </c>
+      <c r="C77" t="s">
+        <v>35</v>
+      </c>
+      <c r="D77" t="s">
+        <v>35</v>
+      </c>
+      <c r="E77" t="s">
+        <v>151</v>
+      </c>
+      <c r="F77" t="s">
+        <v>151</v>
+      </c>
+      <c r="G77" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78">
+        <v>3</v>
+      </c>
+      <c r="B78" t="s">
+        <v>10</v>
+      </c>
+      <c r="C78" t="s">
+        <v>113</v>
+      </c>
+      <c r="D78" t="s">
+        <v>113</v>
+      </c>
+      <c r="E78" t="s">
+        <v>137</v>
+      </c>
+      <c r="F78" t="s">
+        <v>154</v>
+      </c>
+      <c r="G78" t="s">
+        <v>162</v>
+      </c>
+      <c r="H78" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79">
+        <v>3</v>
+      </c>
+      <c r="B79" t="s">
+        <v>10</v>
+      </c>
+      <c r="C79" t="s">
+        <v>37</v>
+      </c>
+      <c r="D79" t="s">
+        <v>37</v>
+      </c>
+      <c r="E79" t="s">
+        <v>138</v>
+      </c>
+      <c r="F79" t="s">
+        <v>138</v>
+      </c>
+      <c r="G79" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80">
+        <v>3</v>
+      </c>
+      <c r="B80" t="s">
+        <v>10</v>
+      </c>
+      <c r="C80" t="s">
+        <v>38</v>
+      </c>
+      <c r="D80" t="s">
+        <v>38</v>
+      </c>
+      <c r="E80" t="s">
+        <v>138</v>
+      </c>
+      <c r="F80" t="s">
+        <v>138</v>
+      </c>
+      <c r="G80" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81">
+        <v>3</v>
+      </c>
+      <c r="B81" t="s">
+        <v>10</v>
+      </c>
+      <c r="C81" t="s">
+        <v>114</v>
+      </c>
+      <c r="D81" t="s">
+        <v>114</v>
+      </c>
+      <c r="F81" t="s">
+        <v>154</v>
+      </c>
+      <c r="G81" t="s">
+        <v>49</v>
+      </c>
+      <c r="H81" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82">
+        <v>3</v>
+      </c>
+      <c r="B82" t="s">
+        <v>10</v>
+      </c>
+      <c r="C82" t="s">
+        <v>115</v>
+      </c>
+      <c r="D82" t="s">
+        <v>115</v>
+      </c>
+      <c r="E82" t="s">
+        <v>134</v>
+      </c>
+      <c r="F82" t="s">
+        <v>154</v>
+      </c>
+      <c r="G82" t="s">
+        <v>162</v>
+      </c>
+      <c r="H82" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83">
+        <v>3</v>
+      </c>
+      <c r="B83" t="s">
+        <v>10</v>
+      </c>
+      <c r="C83" t="s">
+        <v>116</v>
+      </c>
+      <c r="D83" t="s">
+        <v>116</v>
+      </c>
+      <c r="F83" t="s">
+        <v>154</v>
+      </c>
+      <c r="G83" t="s">
+        <v>49</v>
+      </c>
+      <c r="H83" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84">
+        <v>3</v>
+      </c>
+      <c r="B84" t="s">
+        <v>10</v>
+      </c>
+      <c r="C84" t="s">
+        <v>117</v>
+      </c>
+      <c r="D84" t="s">
+        <v>117</v>
+      </c>
+      <c r="E84" t="s">
+        <v>139</v>
+      </c>
+      <c r="F84" t="s">
+        <v>154</v>
+      </c>
+      <c r="G84" t="s">
+        <v>162</v>
+      </c>
+      <c r="H84" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85">
+        <v>3</v>
+      </c>
+      <c r="B85" t="s">
+        <v>10</v>
+      </c>
+      <c r="C85" t="s">
         <v>118</v>
       </c>
-      <c r="F64" t="s">
-        <v>110</v>
-      </c>
-      <c r="G64" t="s">
+      <c r="D85" t="s">
+        <v>118</v>
+      </c>
+      <c r="F85" t="s">
+        <v>154</v>
+      </c>
+      <c r="G85" t="s">
+        <v>49</v>
+      </c>
+      <c r="H85" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86">
+        <v>3</v>
+      </c>
+      <c r="B86" t="s">
+        <v>10</v>
+      </c>
+      <c r="C86" t="s">
+        <v>119</v>
+      </c>
+      <c r="D86" t="s">
+        <v>119</v>
+      </c>
+      <c r="E86" t="s">
+        <v>140</v>
+      </c>
+      <c r="F86" t="s">
+        <v>154</v>
+      </c>
+      <c r="G86" t="s">
+        <v>162</v>
+      </c>
+      <c r="H86" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87">
+        <v>3</v>
+      </c>
+      <c r="B87" t="s">
+        <v>10</v>
+      </c>
+      <c r="C87" t="s">
+        <v>120</v>
+      </c>
+      <c r="D87" t="s">
+        <v>120</v>
+      </c>
+      <c r="E87" t="s">
+        <v>141</v>
+      </c>
+      <c r="F87" t="s">
+        <v>154</v>
+      </c>
+      <c r="G87" t="s">
+        <v>162</v>
+      </c>
+      <c r="H87" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88">
+        <v>3</v>
+      </c>
+      <c r="B88" t="s">
+        <v>10</v>
+      </c>
+      <c r="C88" t="s">
+        <v>121</v>
+      </c>
+      <c r="D88" t="s">
+        <v>121</v>
+      </c>
+      <c r="F88" t="s">
+        <v>154</v>
+      </c>
+      <c r="G88" t="s">
+        <v>49</v>
+      </c>
+      <c r="H88" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89">
+        <v>3</v>
+      </c>
+      <c r="B89" t="s">
+        <v>10</v>
+      </c>
+      <c r="C89" t="s">
+        <v>122</v>
+      </c>
+      <c r="D89" t="s">
+        <v>122</v>
+      </c>
+      <c r="E89" t="s">
+        <v>143</v>
+      </c>
+      <c r="F89" t="s">
+        <v>154</v>
+      </c>
+      <c r="G89" t="s">
+        <v>162</v>
+      </c>
+      <c r="H89" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90">
+        <v>3</v>
+      </c>
+      <c r="B90" t="s">
+        <v>10</v>
+      </c>
+      <c r="C90" t="s">
+        <v>36</v>
+      </c>
+      <c r="D90" t="s">
+        <v>36</v>
+      </c>
+      <c r="E90" t="s">
+        <v>132</v>
+      </c>
+      <c r="F90" t="s">
+        <v>132</v>
+      </c>
+      <c r="G90" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91">
+        <v>3</v>
+      </c>
+      <c r="B91" t="s">
+        <v>10</v>
+      </c>
+      <c r="C91" t="s">
+        <v>123</v>
+      </c>
+      <c r="D91" t="s">
+        <v>123</v>
+      </c>
+      <c r="F91" t="s">
+        <v>154</v>
+      </c>
+      <c r="G91" t="s">
+        <v>49</v>
+      </c>
+      <c r="H91" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92">
+        <v>3</v>
+      </c>
+      <c r="B92" t="s">
+        <v>10</v>
+      </c>
+      <c r="C92" t="s">
+        <v>124</v>
+      </c>
+      <c r="D92" t="s">
+        <v>124</v>
+      </c>
+      <c r="E92" t="s">
+        <v>134</v>
+      </c>
+      <c r="F92" t="s">
+        <v>154</v>
+      </c>
+      <c r="G92" t="s">
+        <v>162</v>
+      </c>
+      <c r="H92" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93">
+        <v>3</v>
+      </c>
+      <c r="B93" t="s">
+        <v>10</v>
+      </c>
+      <c r="C93" t="s">
+        <v>125</v>
+      </c>
+      <c r="D93" t="s">
+        <v>125</v>
+      </c>
+      <c r="E93" t="s">
+        <v>130</v>
+      </c>
+      <c r="F93" t="s">
+        <v>154</v>
+      </c>
+      <c r="G93" t="s">
+        <v>162</v>
+      </c>
+      <c r="H93" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94">
+        <v>3</v>
+      </c>
+      <c r="B94" t="s">
+        <v>10</v>
+      </c>
+      <c r="C94" t="s">
+        <v>126</v>
+      </c>
+      <c r="D94" t="s">
+        <v>126</v>
+      </c>
+      <c r="E94" t="s">
+        <v>152</v>
+      </c>
+      <c r="F94" t="s">
+        <v>154</v>
+      </c>
+      <c r="G94" t="s">
+        <v>162</v>
+      </c>
+      <c r="H94" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95">
+        <v>3</v>
+      </c>
+      <c r="B95" t="s">
+        <v>10</v>
+      </c>
+      <c r="C95" t="s">
+        <v>127</v>
+      </c>
+      <c r="D95" t="s">
+        <v>127</v>
+      </c>
+      <c r="F95" t="s">
+        <v>154</v>
+      </c>
+      <c r="G95" t="s">
+        <v>49</v>
+      </c>
+      <c r="H95" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96">
+        <v>3</v>
+      </c>
+      <c r="B96" t="s">
+        <v>10</v>
+      </c>
+      <c r="C96" t="s">
+        <v>128</v>
+      </c>
+      <c r="D96" t="s">
+        <v>128</v>
+      </c>
+      <c r="E96" t="s">
+        <v>134</v>
+      </c>
+      <c r="F96" t="s">
+        <v>154</v>
+      </c>
+      <c r="G96" t="s">
+        <v>162</v>
+      </c>
+      <c r="H96" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97">
+        <v>3</v>
+      </c>
+      <c r="B97" t="s">
+        <v>10</v>
+      </c>
+      <c r="C97" t="s">
+        <v>129</v>
+      </c>
+      <c r="D97" t="s">
+        <v>129</v>
+      </c>
+      <c r="E97" t="s">
+        <v>153</v>
+      </c>
+      <c r="F97" t="s">
+        <v>154</v>
+      </c>
+      <c r="G97" t="s">
+        <v>162</v>
+      </c>
+      <c r="H97" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98">
+        <v>3</v>
+      </c>
+      <c r="B98" t="s">
+        <v>10</v>
+      </c>
+      <c r="C98" t="s">
+        <v>18</v>
+      </c>
+      <c r="E98" t="s">
+        <v>154</v>
+      </c>
+      <c r="F98" t="s">
+        <v>156</v>
+      </c>
+      <c r="G98" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
-      <c r="A65">
-        <v>3</v>
-      </c>
-      <c r="B65" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" t="s">
+    <row r="99" spans="1:8">
+      <c r="A99">
+        <v>3</v>
+      </c>
+      <c r="B99" t="s">
+        <v>10</v>
+      </c>
+      <c r="C99" t="s">
         <v>25</v>
       </c>
-      <c r="E65" t="s">
-        <v>118</v>
-      </c>
-      <c r="F65" t="s">
-        <v>124</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="E99" t="s">
+        <v>154</v>
+      </c>
+      <c r="F99" t="s">
+        <v>160</v>
+      </c>
+      <c r="G99" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
-      <c r="A66">
-        <v>3</v>
-      </c>
-      <c r="B66" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" t="s">
-        <v>35</v>
-      </c>
-      <c r="E66" t="s">
-        <v>118</v>
-      </c>
-      <c r="F66" t="s">
-        <v>125</v>
-      </c>
-      <c r="G66" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
-      <c r="A67">
-        <v>3</v>
-      </c>
-      <c r="B67" t="s">
-        <v>10</v>
-      </c>
-      <c r="C67" t="s">
-        <v>36</v>
-      </c>
-      <c r="E67" t="s">
-        <v>118</v>
-      </c>
-      <c r="F67" t="s">
-        <v>109</v>
-      </c>
-      <c r="G67" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
-      <c r="A68">
-        <v>3</v>
-      </c>
-      <c r="B68" t="s">
-        <v>10</v>
-      </c>
-      <c r="C68" t="s">
-        <v>37</v>
-      </c>
-      <c r="E68" t="s">
-        <v>118</v>
-      </c>
-      <c r="F68" t="s">
-        <v>102</v>
-      </c>
-      <c r="G68" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69">
-        <v>3</v>
-      </c>
-      <c r="B69" t="s">
-        <v>10</v>
-      </c>
-      <c r="C69" t="s">
-        <v>38</v>
-      </c>
-      <c r="E69" t="s">
-        <v>118</v>
-      </c>
-      <c r="F69" t="s">
-        <v>102</v>
-      </c>
-      <c r="G69" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70">
-        <v>3</v>
-      </c>
-      <c r="B70" t="s">
-        <v>10</v>
-      </c>
-      <c r="C70" t="s">
-        <v>39</v>
-      </c>
-      <c r="E70" t="s">
-        <v>118</v>
-      </c>
-      <c r="F70" t="s">
-        <v>126</v>
-      </c>
-      <c r="G70" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
-      <c r="A71">
-        <v>3</v>
-      </c>
-      <c r="B71" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" t="s">
+    <row r="100" spans="1:8">
+      <c r="A100">
+        <v>3</v>
+      </c>
+      <c r="B100" t="s">
+        <v>10</v>
+      </c>
+      <c r="C100" t="s">
         <v>40</v>
       </c>
-      <c r="E71" t="s">
-        <v>118</v>
-      </c>
-      <c r="F71" t="s">
-        <v>117</v>
-      </c>
-      <c r="G71" t="s">
+      <c r="E100" t="s">
+        <v>154</v>
+      </c>
+      <c r="F100" t="s">
+        <v>161</v>
+      </c>
+      <c r="G100" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance dataset pairing logic to include host titles
- Updated the item_keys function to return multiple identifying values for datasets, including host titles for distributions.
- Modified the pair_items function to allow pairing based on any identifying value (title, name, identifier, licence, host title) instead of just exact matches.
- Added a new test to ensure distributions are correctly paired by host title regardless of their order in the input lists.
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="164">
   <si>
     <t>rda model</t>
   </si>
@@ -169,9 +169,6 @@
     <t>Correct</t>
   </si>
   <si>
-    <t>Mismatch</t>
-  </si>
-  <si>
     <t>Missed</t>
   </si>
   <si>
@@ -229,6 +226,24 @@
     <t>dmp.dataset[0].dataset_id.type</t>
   </si>
   <si>
+    <t>dmp.dataset[0].distribution[1].title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].data_access</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].license_ref</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].license[0].start_date</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.title</t>
+  </si>
+  <si>
+    <t>dmp.dataset[0].distribution[1].host.url</t>
+  </si>
+  <si>
     <t>dmp.dataset[0].distribution[0].title</t>
   </si>
   <si>
@@ -244,24 +259,6 @@
     <t>dmp.dataset[0].distribution[0].host.url</t>
   </si>
   <si>
-    <t>dmp.dataset[0].distribution[1].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].host.title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[0].distribution[1].host.url</t>
-  </si>
-  <si>
     <t>dmp.dataset[0].metadata[0].description</t>
   </si>
   <si>
@@ -487,12 +484,12 @@
     <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
   </si>
   <si>
+    <t>null</t>
+  </si>
+  <si>
     <t>servers at the Rehabilitation Institute of Chicago</t>
   </si>
   <si>
-    <t>null</t>
-  </si>
-  <si>
     <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
   </si>
   <si>
@@ -512,9 +509,6 @@
   </si>
   <si>
     <t>both empty</t>
-  </si>
-  <si>
-    <t>only 0% of the model's words are in the reference</t>
   </si>
 </sst>
 </file>
@@ -921,22 +915,22 @@
         <v>96</v>
       </c>
       <c r="E2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F2">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>0.542</v>
+        <v>0.552</v>
       </c>
       <c r="I2">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="J2">
-        <v>0.671</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -998,13 +992,13 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>25</v>
@@ -1013,16 +1007,16 @@
         <v>96</v>
       </c>
       <c r="I2">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J2">
-        <v>0.542</v>
+        <v>0.552</v>
       </c>
       <c r="K2">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="L2">
-        <v>0.671</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1083,7 +1077,7 @@
         <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1202,7 +1196,7 @@
         <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1457,7 +1451,7 @@
         <v>48</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1484,7 +1478,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1498,19 +1492,19 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1527,10 +1521,10 @@
         <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G2" t="s">
         <v>49</v>
@@ -1544,22 +1538,22 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1570,22 +1564,22 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1596,22 +1590,22 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1622,22 +1616,22 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1648,19 +1642,19 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1671,22 +1665,22 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1697,19 +1691,19 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9" t="s">
         <v>49</v>
       </c>
       <c r="H9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1720,19 +1714,19 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G10" t="s">
         <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1743,19 +1737,19 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G11" t="s">
         <v>49</v>
       </c>
       <c r="H11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1766,22 +1760,22 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1798,10 +1792,10 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G13" t="s">
         <v>49</v>
@@ -1821,10 +1815,10 @@
         <v>17</v>
       </c>
       <c r="E14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G14" t="s">
         <v>49</v>
@@ -1838,22 +1832,22 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1870,10 +1864,10 @@
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G16" t="s">
         <v>49</v>
@@ -1893,10 +1887,10 @@
         <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G17" t="s">
         <v>49</v>
@@ -1910,19 +1904,19 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G18" t="s">
         <v>49</v>
       </c>
       <c r="H18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1933,22 +1927,22 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1959,19 +1953,19 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F20" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1982,22 +1976,22 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2008,19 +2002,19 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F22" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G22" t="s">
         <v>49</v>
       </c>
       <c r="H22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2031,22 +2025,22 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D23" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F23" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H23" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2057,22 +2051,22 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="D24" t="s">
         <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F24" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H24" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2086,16 +2080,16 @@
         <v>74</v>
       </c>
       <c r="D25" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G25" t="s">
         <v>49</v>
       </c>
       <c r="H25" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2109,16 +2103,16 @@
         <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G26" t="s">
         <v>49</v>
       </c>
       <c r="H26" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2132,19 +2126,19 @@
         <v>76</v>
       </c>
       <c r="D27" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F27" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2158,16 +2152,16 @@
         <v>77</v>
       </c>
       <c r="D28" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G28" t="s">
         <v>49</v>
       </c>
       <c r="H28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2181,19 +2175,19 @@
         <v>78</v>
       </c>
       <c r="D29" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H29" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2204,22 +2198,19 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G30" t="s">
-        <v>162</v>
-      </c>
-      <c r="H30" t="s">
-        <v>163</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2230,19 +2221,19 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D31" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="F31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G31" t="s">
         <v>49</v>
       </c>
       <c r="H31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2253,19 +2244,19 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E32" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H32" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2276,22 +2267,22 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F33" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G33" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H33" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2302,19 +2293,19 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F34" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G34" t="s">
         <v>49</v>
       </c>
       <c r="H34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2325,22 +2316,22 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E35" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F35" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G35" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2357,10 +2348,10 @@
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G36" t="s">
         <v>49</v>
@@ -2380,10 +2371,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G37" t="s">
         <v>49</v>
@@ -2397,22 +2388,22 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2429,10 +2420,10 @@
         <v>26</v>
       </c>
       <c r="E39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
         <v>49</v>
@@ -2452,10 +2443,10 @@
         <v>27</v>
       </c>
       <c r="E40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G40" t="s">
         <v>49</v>
@@ -2469,19 +2460,19 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F41" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G41" t="s">
         <v>49</v>
       </c>
       <c r="H41" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2492,22 +2483,22 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E42" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2518,19 +2509,19 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F43" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G43" t="s">
         <v>49</v>
       </c>
       <c r="H43" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2541,22 +2532,22 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F44" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G44" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H44" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2567,19 +2558,19 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G45" t="s">
         <v>49</v>
       </c>
       <c r="H45" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2590,22 +2581,22 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F46" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H46" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2616,22 +2607,22 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E47" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F47" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H47" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2642,19 +2633,19 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F48" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G48" t="s">
         <v>49</v>
       </c>
       <c r="H48" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2665,19 +2656,19 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G49" t="s">
         <v>49</v>
       </c>
       <c r="H49" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2688,22 +2679,22 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D50" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E50" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2714,19 +2705,19 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D51" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F51" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G51" t="s">
         <v>49</v>
       </c>
       <c r="H51" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2737,22 +2728,22 @@
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D52" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E52" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H52" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2763,22 +2754,22 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E53" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F53" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G53" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H53" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2789,19 +2780,19 @@
         <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F54" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G54" t="s">
         <v>49</v>
       </c>
       <c r="H54" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2818,10 +2809,10 @@
         <v>23</v>
       </c>
       <c r="E55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G55" t="s">
         <v>49</v>
@@ -2841,10 +2832,10 @@
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G56" t="s">
         <v>49</v>
@@ -2858,19 +2849,19 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D57" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F57" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G57" t="s">
         <v>49</v>
       </c>
       <c r="H57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2881,22 +2872,22 @@
         <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E58" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F58" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H58" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2913,10 +2904,10 @@
         <v>34</v>
       </c>
       <c r="E59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G59" t="s">
         <v>49</v>
@@ -2936,10 +2927,10 @@
         <v>29</v>
       </c>
       <c r="E60" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F60" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G60" t="s">
         <v>49</v>
@@ -2953,22 +2944,22 @@
         <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D61" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E61" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F61" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H61" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2985,10 +2976,10 @@
         <v>32</v>
       </c>
       <c r="E62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G62" t="s">
         <v>49</v>
@@ -3008,10 +2999,10 @@
         <v>33</v>
       </c>
       <c r="E63" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F63" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G63" t="s">
         <v>49</v>
@@ -3025,19 +3016,19 @@
         <v>10</v>
       </c>
       <c r="C64" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D64" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F64" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G64" t="s">
         <v>49</v>
       </c>
       <c r="H64" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -3048,22 +3039,22 @@
         <v>10</v>
       </c>
       <c r="C65" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D65" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E65" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G65" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -3074,19 +3065,19 @@
         <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F66" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G66" t="s">
         <v>49</v>
       </c>
       <c r="H66" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -3097,22 +3088,22 @@
         <v>10</v>
       </c>
       <c r="C67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F67" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H67" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -3129,10 +3120,10 @@
         <v>30</v>
       </c>
       <c r="E68" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F68" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G68" t="s">
         <v>49</v>
@@ -3146,22 +3137,22 @@
         <v>10</v>
       </c>
       <c r="C69" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D69" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F69" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G69" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -3172,22 +3163,22 @@
         <v>10</v>
       </c>
       <c r="C70" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D70" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E70" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F70" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G70" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -3198,19 +3189,19 @@
         <v>10</v>
       </c>
       <c r="C71" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D71" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F71" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G71" t="s">
         <v>49</v>
       </c>
       <c r="H71" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -3221,22 +3212,22 @@
         <v>10</v>
       </c>
       <c r="C72" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D72" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E72" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G72" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -3253,10 +3244,10 @@
         <v>31</v>
       </c>
       <c r="E73" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F73" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G73" t="s">
         <v>49</v>
@@ -3270,19 +3261,19 @@
         <v>10</v>
       </c>
       <c r="C74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F74" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G74" t="s">
         <v>49</v>
       </c>
       <c r="H74" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -3293,22 +3284,22 @@
         <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D75" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E75" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F75" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G75" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H75" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -3325,10 +3316,10 @@
         <v>39</v>
       </c>
       <c r="E76" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F76" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G76" t="s">
         <v>49</v>
@@ -3348,10 +3339,10 @@
         <v>35</v>
       </c>
       <c r="E77" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F77" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G77" t="s">
         <v>49</v>
@@ -3365,22 +3356,22 @@
         <v>10</v>
       </c>
       <c r="C78" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D78" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E78" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F78" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G78" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H78" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -3397,10 +3388,10 @@
         <v>37</v>
       </c>
       <c r="E79" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F79" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G79" t="s">
         <v>49</v>
@@ -3420,10 +3411,10 @@
         <v>38</v>
       </c>
       <c r="E80" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F80" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G80" t="s">
         <v>49</v>
@@ -3437,19 +3428,19 @@
         <v>10</v>
       </c>
       <c r="C81" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D81" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F81" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G81" t="s">
         <v>49</v>
       </c>
       <c r="H81" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -3460,22 +3451,22 @@
         <v>10</v>
       </c>
       <c r="C82" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D82" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E82" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F82" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G82" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H82" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -3486,19 +3477,19 @@
         <v>10</v>
       </c>
       <c r="C83" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D83" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F83" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G83" t="s">
         <v>49</v>
       </c>
       <c r="H83" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -3509,22 +3500,22 @@
         <v>10</v>
       </c>
       <c r="C84" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D84" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E84" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F84" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G84" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H84" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -3535,19 +3526,19 @@
         <v>10</v>
       </c>
       <c r="C85" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D85" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F85" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G85" t="s">
         <v>49</v>
       </c>
       <c r="H85" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -3558,22 +3549,22 @@
         <v>10</v>
       </c>
       <c r="C86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D86" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E86" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F86" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G86" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H86" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -3584,22 +3575,22 @@
         <v>10</v>
       </c>
       <c r="C87" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D87" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E87" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F87" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G87" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H87" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -3610,19 +3601,19 @@
         <v>10</v>
       </c>
       <c r="C88" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D88" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F88" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G88" t="s">
         <v>49</v>
       </c>
       <c r="H88" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -3633,22 +3624,22 @@
         <v>10</v>
       </c>
       <c r="C89" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D89" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E89" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F89" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G89" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H89" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -3665,10 +3656,10 @@
         <v>36</v>
       </c>
       <c r="E90" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F90" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G90" t="s">
         <v>49</v>
@@ -3682,19 +3673,19 @@
         <v>10</v>
       </c>
       <c r="C91" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D91" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F91" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G91" t="s">
         <v>49</v>
       </c>
       <c r="H91" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3705,22 +3696,22 @@
         <v>10</v>
       </c>
       <c r="C92" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D92" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E92" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F92" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G92" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H92" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -3731,22 +3722,22 @@
         <v>10</v>
       </c>
       <c r="C93" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D93" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E93" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F93" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G93" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H93" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3757,22 +3748,22 @@
         <v>10</v>
       </c>
       <c r="C94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E94" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F94" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G94" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H94" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -3783,19 +3774,19 @@
         <v>10</v>
       </c>
       <c r="C95" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D95" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F95" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G95" t="s">
         <v>49</v>
       </c>
       <c r="H95" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -3806,22 +3797,22 @@
         <v>10</v>
       </c>
       <c r="C96" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D96" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E96" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F96" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G96" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H96" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -3832,22 +3823,22 @@
         <v>10</v>
       </c>
       <c r="C97" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D97" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E97" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F97" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H97" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -3858,16 +3849,16 @@
         <v>10</v>
       </c>
       <c r="C98" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E98" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F98" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G98" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -3878,36 +3869,16 @@
         <v>10</v>
       </c>
       <c r="C99" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E99" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F99" t="s">
         <v>160</v>
       </c>
       <c r="G99" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8">
-      <c r="A100">
-        <v>3</v>
-      </c>
-      <c r="B100" t="s">
-        <v>10</v>
-      </c>
-      <c r="C100" t="s">
-        <v>40</v>
-      </c>
-      <c r="E100" t="s">
-        <v>154</v>
-      </c>
-      <c r="F100" t="s">
-        <v>161</v>
-      </c>
-      <c r="G100" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RDA extraction and field matrix notebooks to version 11
- Changed prompt and schema paths in build_rda_extraction_notebook.py to v11.
- Updated run and prompt variables in build_rda_field_matrix_notebook.py to v11.
- Removed v12 references from build_rda_version_comparison_notebook.py, retaining only v11.
</commit_message>
<xml_diff>
--- a/data/output/5_rda/evaluation/evaluation_results.xlsx
+++ b/data/output/5_rda/evaluation/evaluation_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="162">
   <si>
     <t>rda model</t>
   </si>
@@ -298,24 +298,6 @@
     <t>dmp.dataset[1].distribution[0].host.url</t>
   </si>
   <si>
-    <t>dmp.dataset[1].distribution[1].title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[1].data_access</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[1].license[0].license_ref</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[1].license[0].start_date</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[1].host.title</t>
-  </si>
-  <si>
-    <t>dmp.dataset[1].distribution[1].host.url</t>
-  </si>
-  <si>
     <t>dmp.dataset[1].metadata[0].metadata_standard_id[0].identifier</t>
   </si>
   <si>
@@ -409,90 +391,99 @@
     <t>CPS 2015</t>
   </si>
   <si>
-    <t>2026-10-19T00:00:00Z</t>
+    <t>2026-10-23T00:00:00Z</t>
   </si>
   <si>
     <t>eng</t>
   </si>
   <si>
-    <t>yes</t>
+    <t>unknown</t>
   </si>
   <si>
     <t>other</t>
   </si>
   <si>
+    <t>Data related to proposed experiments</t>
+  </si>
+  <si>
+    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>dataset</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>shared</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>project's website</t>
+  </si>
+  <si>
+    <t>Rehabilitation Institute of Chicago servers</t>
+  </si>
+  <si>
+    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+  </si>
+  <si>
+    <t>Code and results for analyses completed on experimental data</t>
+  </si>
+  <si>
+    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+  </si>
+  <si>
+    <t>GNU Public License</t>
+  </si>
+  <si>
+    <t>labs' websites</t>
+  </si>
+  <si>
+    <t>Simulation code for controller development and testing</t>
+  </si>
+  <si>
+    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
+  </si>
+  <si>
+    <t>Select videos of the experiments</t>
+  </si>
+  <si>
+    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
+  </si>
+  <si>
+    <t>The Data Management Plan should clearly articulate how the PI and co-PIs plan to manage and disseminate data generated by the project.</t>
+  </si>
+  <si>
+    <t>planned</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
     <t>data related to each of our proposed experiments</t>
   </si>
   <si>
-    <t>These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>dataset</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>shared</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>project's website</t>
-  </si>
-  <si>
-    <t>Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>The contents of each data file, including the experimental conditions or the analysis procedures used during generation will be documented.</t>
+    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>servers at the Rehabilitation Institute of Chicago</t>
   </si>
   <si>
     <t>code and results for all analyses completed on experimental data</t>
   </si>
   <si>
-    <t>Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
+    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
   </si>
   <si>
     <t>simulation code for controller development and testing</t>
   </si>
   <si>
-    <t>The proposed foundational developments will produce substantial simulation code for controller development and testing. These and the outputs relevant to all key findings will also be managed.</t>
-  </si>
-  <si>
-    <t>GNU Public License</t>
-  </si>
-  <si>
-    <t>labs' websites</t>
-  </si>
-  <si>
-    <t>select videos of the experiments</t>
-  </si>
-  <si>
-    <t>Select videos of the experiments will be distributed, with subject faces blurred so as to be unidentifiable.</t>
-  </si>
-  <si>
-    <t>The Data Management Plan should clearly articulate how the PI and co-PIs plan to manage and disseminate data generated by the project.</t>
-  </si>
-  <si>
-    <t>planned</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>First, we will have data related to each of our proposed experiments. These will include the detailed protocols used for each experiment, the raw data collected from each experiment, and the experimental code used to collect those data. The relevant code will include both the data acquisition code, and the code for the controllers used in the experiment. Together, this information will be sufficient for recreating the circumstances of each data collection session.</t>
-  </si>
-  <si>
-    <t>null</t>
-  </si>
-  <si>
-    <t>servers at the Rehabilitation Institute of Chicago</t>
-  </si>
-  <si>
-    <t>Our second type of data will be the code and results for all analyses completed on experimental data. Specifically, we store all code necessary to recreate figures, tables, and other results reported in all published manuscripts.</t>
-  </si>
-  <si>
     <t>videos of the experiments</t>
   </si>
   <si>
@@ -509,6 +500,9 @@
   </si>
   <si>
     <t>both empty</t>
+  </si>
+  <si>
+    <t>empty where the reference has a value</t>
   </si>
 </sst>
 </file>
@@ -912,25 +906,25 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E2">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>0.552</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="I2">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="J2">
-        <v>0.6899999999999999</v>
+        <v>0.6889999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -992,31 +986,31 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <v>25</v>
       </c>
       <c r="H2">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="I2">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J2">
-        <v>0.552</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="K2">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="L2">
-        <v>0.6899999999999999</v>
+        <v>0.6889999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +1156,7 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1478,7 +1472,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1521,10 +1515,10 @@
         <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G2" t="s">
         <v>49</v>
@@ -1544,16 +1538,16 @@
         <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1570,16 +1564,16 @@
         <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F4" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1596,16 +1590,16 @@
         <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F5" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1622,16 +1616,16 @@
         <v>59</v>
       </c>
       <c r="E6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="F6" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1648,13 +1642,13 @@
         <v>60</v>
       </c>
       <c r="F7" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1671,16 +1665,16 @@
         <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G8" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1697,13 +1691,13 @@
         <v>62</v>
       </c>
       <c r="F9" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G9" t="s">
         <v>49</v>
       </c>
       <c r="H9" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1720,13 +1714,13 @@
         <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G10" t="s">
         <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1743,13 +1737,13 @@
         <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G11" t="s">
         <v>49</v>
       </c>
       <c r="H11" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1766,16 +1760,16 @@
         <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F12" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G12" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H12" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1792,10 +1786,10 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F13" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="G13" t="s">
         <v>49</v>
@@ -1815,10 +1809,10 @@
         <v>17</v>
       </c>
       <c r="E14" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F14" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G14" t="s">
         <v>49</v>
@@ -1838,16 +1832,16 @@
         <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G15" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1864,10 +1858,10 @@
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F16" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G16" t="s">
         <v>49</v>
@@ -1887,10 +1881,10 @@
         <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F17" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G17" t="s">
         <v>49</v>
@@ -1910,13 +1904,13 @@
         <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G18" t="s">
         <v>49</v>
       </c>
       <c r="H18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1933,16 +1927,16 @@
         <v>68</v>
       </c>
       <c r="E19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F19" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G19" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H19" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1959,13 +1953,13 @@
         <v>75</v>
       </c>
       <c r="F20" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1982,16 +1976,16 @@
         <v>76</v>
       </c>
       <c r="E21" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F21" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G21" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H21" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -2008,13 +2002,13 @@
         <v>77</v>
       </c>
       <c r="F22" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G22" t="s">
         <v>49</v>
       </c>
       <c r="H22" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -2031,16 +2025,16 @@
         <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F23" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G23" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H23" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2057,16 +2051,16 @@
         <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F24" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G24" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H24" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -2083,13 +2077,13 @@
         <v>79</v>
       </c>
       <c r="F25" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G25" t="s">
         <v>49</v>
       </c>
       <c r="H25" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2106,13 +2100,13 @@
         <v>69</v>
       </c>
       <c r="F26" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G26" t="s">
         <v>49</v>
       </c>
       <c r="H26" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2129,16 +2123,16 @@
         <v>70</v>
       </c>
       <c r="E27" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F27" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G27" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H27" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -2155,13 +2149,13 @@
         <v>71</v>
       </c>
       <c r="F28" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G28" t="s">
         <v>49</v>
       </c>
       <c r="H28" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2178,16 +2172,16 @@
         <v>72</v>
       </c>
       <c r="E29" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F29" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G29" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H29" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2204,10 +2198,10 @@
         <v>73</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F30" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="G30" t="s">
         <v>49</v>
@@ -2227,13 +2221,13 @@
         <v>74</v>
       </c>
       <c r="F31" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G31" t="s">
         <v>49</v>
       </c>
       <c r="H31" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2250,13 +2244,13 @@
         <v>80</v>
       </c>
       <c r="E32" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="G32" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H32" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -2273,16 +2267,16 @@
         <v>81</v>
       </c>
       <c r="E33" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F33" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G33" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H33" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2299,13 +2293,13 @@
         <v>82</v>
       </c>
       <c r="F34" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G34" t="s">
         <v>49</v>
       </c>
       <c r="H34" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2322,16 +2316,16 @@
         <v>83</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F35" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G35" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H35" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2348,10 +2342,10 @@
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F36" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="G36" t="s">
         <v>49</v>
@@ -2371,10 +2365,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="F37" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="G37" t="s">
         <v>49</v>
@@ -2394,16 +2388,16 @@
         <v>84</v>
       </c>
       <c r="E38" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F38" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2420,10 +2414,10 @@
         <v>26</v>
       </c>
       <c r="E39" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G39" t="s">
         <v>49</v>
@@ -2443,10 +2437,10 @@
         <v>27</v>
       </c>
       <c r="E40" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G40" t="s">
         <v>49</v>
@@ -2466,13 +2460,13 @@
         <v>85</v>
       </c>
       <c r="F41" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G41" t="s">
         <v>49</v>
       </c>
       <c r="H41" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2489,16 +2483,16 @@
         <v>86</v>
       </c>
       <c r="E42" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F42" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G42" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H42" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2515,13 +2509,13 @@
         <v>87</v>
       </c>
       <c r="F43" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G43" t="s">
         <v>49</v>
       </c>
       <c r="H43" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2538,16 +2532,16 @@
         <v>88</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F44" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G44" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H44" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2563,14 +2557,17 @@
       <c r="D45" t="s">
         <v>89</v>
       </c>
+      <c r="E45" t="s">
+        <v>139</v>
+      </c>
       <c r="F45" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G45" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="H45" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2587,16 +2584,16 @@
         <v>90</v>
       </c>
       <c r="E46" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F46" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G46" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H46" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2616,13 +2613,13 @@
         <v>140</v>
       </c>
       <c r="F47" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G47" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H47" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2639,13 +2636,13 @@
         <v>92</v>
       </c>
       <c r="F48" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G48" t="s">
         <v>49</v>
       </c>
       <c r="H48" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2656,19 +2653,19 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="D49" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="F49" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="G49" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="H49" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2679,22 +2676,19 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="D50" t="s">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="F50" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="G50" t="s">
-        <v>161</v>
-      </c>
-      <c r="H50" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2705,19 +2699,19 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D51" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F51" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G51" t="s">
         <v>49</v>
       </c>
       <c r="H51" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2728,22 +2722,22 @@
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D52" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E52" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="F52" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G52" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H52" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2754,22 +2748,19 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="D53" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E53" t="s">
         <v>141</v>
       </c>
       <c r="F53" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G53" t="s">
-        <v>161</v>
-      </c>
-      <c r="H53" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2780,19 +2771,19 @@
         <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="D54" t="s">
-        <v>98</v>
+        <v>29</v>
+      </c>
+      <c r="E54" t="s">
+        <v>142</v>
       </c>
       <c r="F54" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="G54" t="s">
         <v>49</v>
-      </c>
-      <c r="H54" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2803,19 +2794,22 @@
         <v>10</v>
       </c>
       <c r="C55" t="s">
-        <v>23</v>
+        <v>95</v>
       </c>
       <c r="D55" t="s">
-        <v>23</v>
+        <v>95</v>
       </c>
       <c r="E55" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F55" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G55" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H55" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2826,10 +2820,10 @@
         <v>10</v>
       </c>
       <c r="C56" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D56" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E56" t="s">
         <v>131</v>
@@ -2849,19 +2843,19 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="D57" t="s">
-        <v>99</v>
+        <v>33</v>
+      </c>
+      <c r="E57" t="s">
+        <v>131</v>
       </c>
       <c r="F57" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="G57" t="s">
         <v>49</v>
-      </c>
-      <c r="H57" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2872,22 +2866,19 @@
         <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D58" t="s">
-        <v>100</v>
-      </c>
-      <c r="E58" t="s">
-        <v>133</v>
+        <v>96</v>
       </c>
       <c r="F58" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G58" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="H58" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2898,19 +2889,22 @@
         <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D59" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="E59" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="F59" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G59" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H59" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2921,19 +2915,19 @@
         <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="D60" t="s">
-        <v>29</v>
-      </c>
-      <c r="E60" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
       <c r="F60" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G60" t="s">
         <v>49</v>
+      </c>
+      <c r="H60" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2944,22 +2938,22 @@
         <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D61" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E61" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F61" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G61" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H61" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2970,16 +2964,16 @@
         <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D62" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G62" t="s">
         <v>49</v>
@@ -2993,19 +2987,22 @@
         <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="D63" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="E63" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F63" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="G63" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H63" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -3016,19 +3013,22 @@
         <v>10</v>
       </c>
       <c r="C64" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D64" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="E64" t="s">
+        <v>140</v>
       </c>
       <c r="F64" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G64" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="H64" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -3039,22 +3039,19 @@
         <v>10</v>
       </c>
       <c r="C65" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D65" t="s">
-        <v>103</v>
-      </c>
-      <c r="E65" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="F65" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G65" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="H65" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -3065,19 +3062,19 @@
         <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D66" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F66" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G66" t="s">
         <v>49</v>
       </c>
       <c r="H66" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -3088,22 +3085,19 @@
         <v>10</v>
       </c>
       <c r="C67" t="s">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="D67" t="s">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="E67" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="F67" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="G67" t="s">
-        <v>161</v>
-      </c>
-      <c r="H67" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -3114,19 +3108,19 @@
         <v>10</v>
       </c>
       <c r="C68" t="s">
-        <v>30</v>
+        <v>104</v>
       </c>
       <c r="D68" t="s">
-        <v>30</v>
-      </c>
-      <c r="E68" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="F68" t="s">
         <v>147</v>
       </c>
       <c r="G68" t="s">
         <v>49</v>
+      </c>
+      <c r="H68" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -3137,22 +3131,22 @@
         <v>10</v>
       </c>
       <c r="C69" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D69" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E69" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="F69" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G69" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H69" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -3163,22 +3157,19 @@
         <v>10</v>
       </c>
       <c r="C70" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="D70" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="E70" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F70" t="s">
         <v>155</v>
       </c>
       <c r="G70" t="s">
-        <v>161</v>
-      </c>
-      <c r="H70" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -3189,19 +3180,19 @@
         <v>10</v>
       </c>
       <c r="C71" t="s">
-        <v>108</v>
+        <v>35</v>
       </c>
       <c r="D71" t="s">
-        <v>108</v>
+        <v>35</v>
+      </c>
+      <c r="E71" t="s">
+        <v>144</v>
       </c>
       <c r="F71" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="G71" t="s">
         <v>49</v>
-      </c>
-      <c r="H71" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -3212,22 +3203,22 @@
         <v>10</v>
       </c>
       <c r="C72" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D72" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E72" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F72" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G72" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H72" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -3238,10 +3229,10 @@
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D73" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E73" t="s">
         <v>131</v>
@@ -3261,19 +3252,19 @@
         <v>10</v>
       </c>
       <c r="C74" t="s">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="D74" t="s">
-        <v>110</v>
+        <v>38</v>
+      </c>
+      <c r="E74" t="s">
+        <v>131</v>
       </c>
       <c r="F74" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="G74" t="s">
         <v>49</v>
-      </c>
-      <c r="H74" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -3284,22 +3275,19 @@
         <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D75" t="s">
-        <v>111</v>
-      </c>
-      <c r="E75" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="F75" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G75" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="H75" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -3310,19 +3298,22 @@
         <v>10</v>
       </c>
       <c r="C76" t="s">
-        <v>39</v>
+        <v>108</v>
       </c>
       <c r="D76" t="s">
-        <v>39</v>
+        <v>108</v>
       </c>
       <c r="E76" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="F76" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="G76" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H76" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -3333,19 +3324,19 @@
         <v>10</v>
       </c>
       <c r="C77" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
       <c r="D77" t="s">
-        <v>35</v>
-      </c>
-      <c r="E77" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="F77" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G77" t="s">
         <v>49</v>
+      </c>
+      <c r="H77" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -3356,22 +3347,22 @@
         <v>10</v>
       </c>
       <c r="C78" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D78" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E78" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F78" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G78" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H78" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -3382,19 +3373,19 @@
         <v>10</v>
       </c>
       <c r="C79" t="s">
-        <v>37</v>
+        <v>111</v>
       </c>
       <c r="D79" t="s">
-        <v>37</v>
-      </c>
-      <c r="E79" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F79" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="G79" t="s">
         <v>49</v>
+      </c>
+      <c r="H79" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -3405,19 +3396,22 @@
         <v>10</v>
       </c>
       <c r="C80" t="s">
-        <v>38</v>
+        <v>112</v>
       </c>
       <c r="D80" t="s">
-        <v>38</v>
+        <v>112</v>
       </c>
       <c r="E80" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F80" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="G80" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H80" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -3434,13 +3428,13 @@
         <v>113</v>
       </c>
       <c r="F81" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G81" t="s">
         <v>49</v>
       </c>
       <c r="H81" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -3456,17 +3450,14 @@
       <c r="D82" t="s">
         <v>114</v>
       </c>
-      <c r="E82" t="s">
-        <v>133</v>
-      </c>
       <c r="F82" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G82" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="H82" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -3483,13 +3474,13 @@
         <v>115</v>
       </c>
       <c r="F83" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G83" t="s">
         <v>49</v>
       </c>
       <c r="H83" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -3500,22 +3491,19 @@
         <v>10</v>
       </c>
       <c r="C84" t="s">
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="D84" t="s">
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="E84" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="F84" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="G84" t="s">
-        <v>161</v>
-      </c>
-      <c r="H84" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -3526,19 +3514,19 @@
         <v>10</v>
       </c>
       <c r="C85" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D85" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F85" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G85" t="s">
         <v>49</v>
       </c>
       <c r="H85" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -3549,22 +3537,22 @@
         <v>10</v>
       </c>
       <c r="C86" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D86" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E86" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="F86" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G86" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H86" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -3575,22 +3563,22 @@
         <v>10</v>
       </c>
       <c r="C87" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D87" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E87" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="F87" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G87" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H87" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -3601,19 +3589,22 @@
         <v>10</v>
       </c>
       <c r="C88" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D88" t="s">
-        <v>120</v>
+        <v>119</v>
+      </c>
+      <c r="E88" t="s">
+        <v>145</v>
       </c>
       <c r="F88" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G88" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="H88" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -3624,22 +3615,19 @@
         <v>10</v>
       </c>
       <c r="C89" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D89" t="s">
-        <v>121</v>
-      </c>
-      <c r="E89" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="F89" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G89" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="H89" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -3650,19 +3638,22 @@
         <v>10</v>
       </c>
       <c r="C90" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="D90" t="s">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="E90" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F90" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="G90" t="s">
-        <v>49</v>
+        <v>158</v>
+      </c>
+      <c r="H90" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -3678,14 +3669,17 @@
       <c r="D91" t="s">
         <v>122</v>
       </c>
+      <c r="E91" t="s">
+        <v>146</v>
+      </c>
       <c r="F91" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G91" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
       <c r="H91" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3696,22 +3690,16 @@
         <v>10</v>
       </c>
       <c r="C92" t="s">
-        <v>123</v>
-      </c>
-      <c r="D92" t="s">
-        <v>123</v>
+        <v>23</v>
       </c>
       <c r="E92" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F92" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="G92" t="s">
-        <v>161</v>
-      </c>
-      <c r="H92" t="s">
-        <v>162</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -3722,22 +3710,16 @@
         <v>10</v>
       </c>
       <c r="C93" t="s">
-        <v>124</v>
-      </c>
-      <c r="D93" t="s">
-        <v>124</v>
+        <v>25</v>
       </c>
       <c r="E93" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="F93" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G93" t="s">
-        <v>161</v>
-      </c>
-      <c r="H93" t="s">
-        <v>162</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3748,136 +3730,15 @@
         <v>10</v>
       </c>
       <c r="C94" t="s">
-        <v>125</v>
-      </c>
-      <c r="D94" t="s">
-        <v>125</v>
+        <v>40</v>
       </c>
       <c r="E94" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F94" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G94" t="s">
-        <v>161</v>
-      </c>
-      <c r="H94" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8">
-      <c r="A95">
-        <v>3</v>
-      </c>
-      <c r="B95" t="s">
-        <v>10</v>
-      </c>
-      <c r="C95" t="s">
-        <v>126</v>
-      </c>
-      <c r="D95" t="s">
-        <v>126</v>
-      </c>
-      <c r="F95" t="s">
-        <v>153</v>
-      </c>
-      <c r="G95" t="s">
-        <v>49</v>
-      </c>
-      <c r="H95" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="96" spans="1:8">
-      <c r="A96">
-        <v>3</v>
-      </c>
-      <c r="B96" t="s">
-        <v>10</v>
-      </c>
-      <c r="C96" t="s">
-        <v>127</v>
-      </c>
-      <c r="D96" t="s">
-        <v>127</v>
-      </c>
-      <c r="E96" t="s">
-        <v>133</v>
-      </c>
-      <c r="F96" t="s">
-        <v>153</v>
-      </c>
-      <c r="G96" t="s">
-        <v>161</v>
-      </c>
-      <c r="H96" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="97" spans="1:8">
-      <c r="A97">
-        <v>3</v>
-      </c>
-      <c r="B97" t="s">
-        <v>10</v>
-      </c>
-      <c r="C97" t="s">
-        <v>128</v>
-      </c>
-      <c r="D97" t="s">
-        <v>128</v>
-      </c>
-      <c r="E97" t="s">
-        <v>152</v>
-      </c>
-      <c r="F97" t="s">
-        <v>153</v>
-      </c>
-      <c r="G97" t="s">
-        <v>161</v>
-      </c>
-      <c r="H97" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8">
-      <c r="A98">
-        <v>3</v>
-      </c>
-      <c r="B98" t="s">
-        <v>10</v>
-      </c>
-      <c r="C98" t="s">
-        <v>25</v>
-      </c>
-      <c r="E98" t="s">
-        <v>153</v>
-      </c>
-      <c r="F98" t="s">
-        <v>159</v>
-      </c>
-      <c r="G98" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8">
-      <c r="A99">
-        <v>3</v>
-      </c>
-      <c r="B99" t="s">
-        <v>10</v>
-      </c>
-      <c r="C99" t="s">
-        <v>40</v>
-      </c>
-      <c r="E99" t="s">
-        <v>153</v>
-      </c>
-      <c r="F99" t="s">
-        <v>160</v>
-      </c>
-      <c r="G99" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>